<commit_message>
Scale user growth to hit ~100K at Year 2 end per pitch deck
Sleeper hit 1M users in first calendar year (2019) — 100K is very
achievable for a focused NHL-only platform with ML moat. Adjusted
Season 2 acquisition (Oct 2027-Mar 2028) to 13-20K new users/month
to account for churn and hit the 100K gate.

Updated model results:
- Y1 End: 10,496 users | $77.5K revenue
- Y2 End: 98,320 users | $1.06M revenue
- 24-month cumulative: $1.14M revenue, $832K net
- Breakeven: Month 10

https://claude.ai/code/session_01W6kNMkpS7XiGU5R6Nuc7yU
</commit_message>
<xml_diff>
--- a/docs/Citrus_Business_Model.xlsx
+++ b/docs/Citrus_Business_Model.xlsx
@@ -1507,73 +1507,73 @@
         <v>150</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="H5" s="13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>2200</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>1800</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M5" s="13" t="n">
         <v>1200</v>
       </c>
-      <c r="I5" s="13" t="n">
-        <v>1800</v>
-      </c>
-      <c r="J5" s="13" t="n">
+      <c r="N5" s="13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="O5" s="13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="P5" s="13" t="n">
+        <v>900</v>
+      </c>
+      <c r="Q5" s="13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="R5" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="K5" s="13" t="n">
-        <v>1500</v>
-      </c>
-      <c r="L5" s="13" t="n">
-        <v>1200</v>
-      </c>
-      <c r="M5" s="13" t="n">
-        <v>1000</v>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>800</v>
-      </c>
-      <c r="O5" s="13" t="n">
-        <v>600</v>
-      </c>
-      <c r="P5" s="13" t="n">
-        <v>500</v>
-      </c>
-      <c r="Q5" s="13" t="n">
-        <v>700</v>
-      </c>
-      <c r="R5" s="13" t="n">
-        <v>900</v>
-      </c>
       <c r="S5" s="13" t="n">
-        <v>1500</v>
+        <v>3500</v>
       </c>
       <c r="T5" s="13" t="n">
-        <v>8000</v>
+        <v>17000</v>
       </c>
       <c r="U5" s="13" t="n">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="V5" s="13" t="n">
-        <v>12000</v>
+        <v>20000</v>
       </c>
       <c r="W5" s="13" t="n">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="X5" s="13" t="n">
-        <v>8000</v>
+        <v>16000</v>
       </c>
       <c r="Y5" s="13" t="n">
-        <v>7000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="7">
@@ -1586,73 +1586,73 @@
         <v>150</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>304.92</v>
+        <v>324.92</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>453.9373759999999</v>
+        <v>520.5933759999999</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>598.0390467327999</v>
+        <v>733.5501635328</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>748.0469181190757</v>
+        <v>1010.900576190116</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>922.9734734095662</v>
+        <v>1341.877999851129</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>1996.156918163092</v>
+        <v>3157.503962671583</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>3521.884957607483</v>
+        <v>5223.662918200508</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>5037.977964432214</v>
+        <v>6705.931633239758</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>5845.759792119227</v>
+        <v>7584.536626832615</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>6242.552396682046</v>
+        <v>8042.421294305813</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>6384.825697377933</v>
+        <v>8137.392608468194</v>
       </c>
       <c r="N7" s="13" t="n">
-        <v>6048.326723244661</v>
+        <v>7888.936724160856</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>5571.724566507111</v>
+        <v>7484.705987260223</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>5079.957593668845</v>
+        <v>7052.428321527902</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>4875.725141995791</v>
+        <v>6997.096080295936</v>
       </c>
       <c r="R7" s="13" t="n">
-        <v>4907.84606672054</v>
+        <v>7751.612978003259</v>
       </c>
       <c r="S7" s="13" t="n">
-        <v>5534.249466844283</v>
+        <v>9871.825867918678</v>
       </c>
       <c r="T7" s="13" t="n">
-        <v>12504.87906601124</v>
+        <v>25035.66625648581</v>
       </c>
       <c r="U7" s="13" t="n">
-        <v>20178.97155973315</v>
+        <v>40379.03233277945</v>
       </c>
       <c r="V7" s="13" t="n">
-        <v>28425.68284962279</v>
+        <v>52868.53231888247</v>
       </c>
       <c r="W7" s="13" t="n">
-        <v>33138.50583959294</v>
+        <v>61034.98530757033</v>
       </c>
       <c r="X7" s="13" t="n">
-        <v>34974.74375342866</v>
+        <v>65682.47804036226</v>
       </c>
       <c r="Y7" s="13" t="n">
-        <v>35469.44141529093</v>
+        <v>66465.53712485488</v>
       </c>
     </row>
     <row r="8">
@@ -1668,70 +1668,70 @@
         <v>2.1</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>6.116880000000001</v>
+        <v>6.39688</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>11.737977664</v>
+        <v>12.917561664</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>18.7019669985792</v>
+        <v>21.6371565537792</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>26.93038781241676</v>
+        <v>33.19330583398732</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>84.00050112472279</v>
+        <v>116.4038875912489</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>206.3983669240087</v>
+        <v>310.6704817359088</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>420.0211845763199</v>
+        <v>627.3344263131045</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>720.6129489524967</v>
+        <v>1024.714742154685</v>
       </c>
       <c r="L8" s="13" t="n">
-        <v>1060.071297897908</v>
+        <v>1461.551959958952</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>1410.949246972961</v>
+        <v>1909.762423101861</v>
       </c>
       <c r="N8" s="13" t="n">
-        <v>1382.10150267852</v>
+        <v>1859.613569715938</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>1349.31251026848</v>
+        <v>1810.016549281564</v>
       </c>
       <c r="P8" s="13" t="n">
-        <v>1309.972949499419</v>
+        <v>1757.478095087501</v>
       </c>
       <c r="Q8" s="13" t="n">
-        <v>1264.535262620204</v>
+        <v>1701.734146750615</v>
       </c>
       <c r="R8" s="13" t="n">
-        <v>1220.056984229687</v>
+        <v>1651.462162907052</v>
       </c>
       <c r="S8" s="13" t="n">
-        <v>1181.622759589976</v>
+        <v>1623.822188874277</v>
       </c>
       <c r="T8" s="13" t="n">
-        <v>1682.248546423961</v>
+        <v>2536.180062243255</v>
       </c>
       <c r="U8" s="13" t="n">
-        <v>2852.941632102115</v>
+        <v>4913.263819145619</v>
       </c>
       <c r="V8" s="13" t="n">
-        <v>4736.542151231612</v>
+        <v>8714.257467324958</v>
       </c>
       <c r="W8" s="13" t="n">
-        <v>7361.223067295005</v>
+        <v>13599.67186820133</v>
       </c>
       <c r="X8" s="13" t="n">
-        <v>10347.48622272291</v>
+        <v>19098.14853892273</v>
       </c>
       <c r="Y8" s="13" t="n">
-        <v>13396.08640540343</v>
+        <v>24836.78792336169</v>
       </c>
     </row>
     <row r="9">
@@ -1747,70 +1747,70 @@
         <v>0.48</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>1.417344</v>
+        <v>1.481344</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>2.7565560832</v>
+        <v>3.0287352832</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>4.44975654608896</v>
+        <v>5.13379698384896</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>6.487526160382886</v>
+        <v>7.957975068949414</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>19.61615602347107</v>
+        <v>27.08206889008193</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>47.87041174443282</v>
+        <v>71.87307423030069</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>97.38879484036977</v>
+        <v>145.2969933966305</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>167.5009576571844</v>
+        <v>238.2299840803673</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>247.4923747222717</v>
+        <v>341.4915619047478</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>331.1978198664364</v>
+        <v>448.7651394951328</v>
       </c>
       <c r="N9" s="13" t="n">
-        <v>343.010948461389</v>
+        <v>461.6882839863314</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>351.8600329239458</v>
+        <v>472.08684161239</v>
       </c>
       <c r="P9" s="13" t="n">
-        <v>357.1415776890728</v>
+        <v>479.2281302069602</v>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>359.0499970359601</v>
+        <v>483.2044497195707</v>
       </c>
       <c r="R9" s="13" t="n">
-        <v>359.580348125058</v>
+        <v>486.5306702237807</v>
       </c>
       <c r="S9" s="13" t="n">
-        <v>360.2609966753766</v>
+        <v>494.1178944738978</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>500.6792073632878</v>
+        <v>748.3042455458548</v>
       </c>
       <c r="U9" s="13" t="n">
-        <v>825.7939619615094</v>
+        <v>1405.559628332325</v>
       </c>
       <c r="V9" s="13" t="n">
-        <v>1349.981345025267</v>
+        <v>2460.654510609062</v>
       </c>
       <c r="W9" s="13" t="n">
-        <v>2083.72524833945</v>
+        <v>3826.588520453663</v>
       </c>
       <c r="X9" s="13" t="n">
-        <v>2926.371774799974</v>
+        <v>5378.86841074672</v>
       </c>
       <c r="Y9" s="13" t="n">
-        <v>3797.530561772548</v>
+        <v>7017.823607567832</v>
       </c>
     </row>
     <row r="10">
@@ -1823,73 +1823,73 @@
         <v>150</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>307.5</v>
+        <v>327.5</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>461.4715999999999</v>
+        <v>528.4716</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>612.53358048</v>
+        <v>749.49646048</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>771.1986416637438</v>
+        <v>1037.671529727744</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>956.3913873823658</v>
+        <v>1383.029280754065</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>2099.773575311286</v>
+        <v>3300.989919152914</v>
       </c>
       <c r="I10" s="15" t="n">
-        <v>3776.153736275925</v>
+        <v>5606.206474166717</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>5555.387943848904</v>
+        <v>7478.563052949494</v>
       </c>
       <c r="K10" s="15" t="n">
-        <v>6733.873698728908</v>
+        <v>8847.481353067669</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>7550.116069302226</v>
+        <v>9845.464816169513</v>
       </c>
       <c r="M10" s="15" t="n">
-        <v>8126.97276421733</v>
+        <v>10495.92017106519</v>
       </c>
       <c r="N10" s="15" t="n">
-        <v>7773.43917438457</v>
+        <v>10210.23857786313</v>
       </c>
       <c r="O10" s="15" t="n">
-        <v>7272.897109699538</v>
+        <v>9766.809378154177</v>
       </c>
       <c r="P10" s="15" t="n">
-        <v>6747.072120857337</v>
+        <v>9289.134546822364</v>
       </c>
       <c r="Q10" s="15" t="n">
-        <v>6499.310401651955</v>
+        <v>9182.034676766121</v>
       </c>
       <c r="R10" s="15" t="n">
-        <v>6487.483399075284</v>
+        <v>9889.605811134092</v>
       </c>
       <c r="S10" s="15" t="n">
-        <v>7076.133223109636</v>
+        <v>11989.76595126685</v>
       </c>
       <c r="T10" s="15" t="n">
-        <v>14687.80681979849</v>
+        <v>28320.15056427492</v>
       </c>
       <c r="U10" s="15" t="n">
-        <v>23857.70715379678</v>
+        <v>46697.85578025739</v>
       </c>
       <c r="V10" s="15" t="n">
-        <v>34512.20634587967</v>
+        <v>64043.44429681649</v>
       </c>
       <c r="W10" s="15" t="n">
-        <v>42583.45415522739</v>
+        <v>78461.24569622532</v>
       </c>
       <c r="X10" s="15" t="n">
-        <v>48248.60175095154</v>
+        <v>90159.4949900317</v>
       </c>
       <c r="Y10" s="15" t="n">
-        <v>52663.05838246691</v>
+        <v>98320.14865578439</v>
       </c>
     </row>
     <row r="12">
@@ -2424,73 +2424,73 @@
         <v>0</v>
       </c>
       <c r="C20" s="19" t="n">
-        <v>0.8390243902439025</v>
+        <v>0.7877862595419848</v>
       </c>
       <c r="D20" s="19" t="n">
-        <v>1.632651716812043</v>
+        <v>1.490756362309725</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>2.366324754936969</v>
+        <v>2.127601368122207</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>3.002044128957727</v>
+        <v>2.579906335548409</v>
       </c>
       <c r="G20" s="19" t="n">
-        <v>3.49416718026541</v>
+        <v>2.975445384677606</v>
       </c>
       <c r="H20" s="19" t="n">
-        <v>4.934658592073812</v>
+        <v>4.346755367194566</v>
       </c>
       <c r="I20" s="19" t="n">
-        <v>6.733538844718849</v>
+        <v>6.823572369818383</v>
       </c>
       <c r="J20" s="19" t="n">
-        <v>9.313660623639826</v>
+        <v>10.33128174810286</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>13.18875206669413</v>
+        <v>14.27462433472272</v>
       </c>
       <c r="L20" s="19" t="n">
-        <v>17.3184578967807</v>
+        <v>18.31344233644008</v>
       </c>
       <c r="M20" s="19" t="n">
-        <v>21.43660520815311</v>
+        <v>22.47089844584475</v>
       </c>
       <c r="N20" s="19" t="n">
-        <v>22.19239660129569</v>
+        <v>22.73504028333967</v>
       </c>
       <c r="O20" s="19" t="n">
-        <v>23.39057623850677</v>
+        <v>23.36590489826112</v>
       </c>
       <c r="P20" s="19" t="n">
-        <v>24.70871064257507</v>
+        <v>24.07873644224043</v>
       </c>
       <c r="Q20" s="19" t="n">
-        <v>24.98088503733397</v>
+        <v>23.79579987863554</v>
       </c>
       <c r="R20" s="19" t="n">
-        <v>24.34899999250717</v>
+        <v>21.6185849462655</v>
       </c>
       <c r="S20" s="19" t="n">
-        <v>21.78991982838567</v>
+        <v>17.66456569675066</v>
       </c>
       <c r="T20" s="19" t="n">
-        <v>14.86217636553309</v>
+        <v>11.59769366456828</v>
       </c>
       <c r="U20" s="19" t="n">
-        <v>15.41948507603415</v>
+        <v>13.53129247992019</v>
       </c>
       <c r="V20" s="19" t="n">
-        <v>17.63585739856222</v>
+        <v>17.4489553156177</v>
       </c>
       <c r="W20" s="19" t="n">
-        <v>22.17985483564871</v>
+        <v>22.21002258379049</v>
       </c>
       <c r="X20" s="19" t="n">
-        <v>27.51138378276651</v>
+        <v>27.14857370527164</v>
       </c>
       <c r="Y20" s="19" t="n">
-        <v>32.64834495996579</v>
+        <v>32.39886428818519</v>
       </c>
     </row>
   </sheetData>
@@ -2723,70 +2723,70 @@
         <v>10</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>419</v>
+        <v>581</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>1030</v>
+        <v>1550</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>2096</v>
+        <v>3130</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>3596</v>
+        <v>5113</v>
       </c>
       <c r="L6" s="13" t="n">
-        <v>5290</v>
+        <v>7293</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>7041</v>
+        <v>9530</v>
       </c>
       <c r="N6" s="13" t="n">
-        <v>6897</v>
+        <v>9279</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>6733</v>
+        <v>9032</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>6537</v>
+        <v>8770</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>6310</v>
+        <v>8492</v>
       </c>
       <c r="R6" s="13" t="n">
-        <v>6088</v>
+        <v>8241</v>
       </c>
       <c r="S6" s="13" t="n">
-        <v>5896</v>
+        <v>8103</v>
       </c>
       <c r="T6" s="13" t="n">
-        <v>8394</v>
+        <v>12656</v>
       </c>
       <c r="U6" s="13" t="n">
-        <v>14236</v>
+        <v>24517</v>
       </c>
       <c r="V6" s="13" t="n">
-        <v>23635</v>
+        <v>43484</v>
       </c>
       <c r="W6" s="13" t="n">
-        <v>36733</v>
+        <v>67862</v>
       </c>
       <c r="X6" s="13" t="n">
-        <v>51634</v>
+        <v>95300</v>
       </c>
       <c r="Y6" s="13" t="n">
-        <v>66846</v>
+        <v>123936</v>
       </c>
     </row>
     <row r="7">
@@ -2802,70 +2802,70 @@
         <v>5</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>196</v>
+        <v>271</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>478</v>
+        <v>718</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>973</v>
+        <v>1452</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>1673</v>
+        <v>2380</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>2472</v>
+        <v>3412</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>3309</v>
+        <v>4483</v>
       </c>
       <c r="N7" s="13" t="n">
-        <v>3427</v>
+        <v>4612</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>3515</v>
+        <v>4716</v>
       </c>
       <c r="P7" s="13" t="n">
-        <v>3568</v>
+        <v>4787</v>
       </c>
       <c r="Q7" s="13" t="n">
-        <v>3587</v>
+        <v>4827</v>
       </c>
       <c r="R7" s="13" t="n">
-        <v>3592</v>
+        <v>4860</v>
       </c>
       <c r="S7" s="13" t="n">
-        <v>3599</v>
+        <v>4936</v>
       </c>
       <c r="T7" s="13" t="n">
-        <v>5002</v>
+        <v>7476</v>
       </c>
       <c r="U7" s="13" t="n">
-        <v>8250</v>
+        <v>14042</v>
       </c>
       <c r="V7" s="13" t="n">
-        <v>13486</v>
+        <v>24582</v>
       </c>
       <c r="W7" s="13" t="n">
-        <v>20816</v>
+        <v>38228</v>
       </c>
       <c r="X7" s="13" t="n">
-        <v>29234</v>
+        <v>53735</v>
       </c>
       <c r="Y7" s="13" t="n">
-        <v>37937</v>
+        <v>70108</v>
       </c>
     </row>
     <row r="8">
@@ -2881,70 +2881,70 @@
         <v>15</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>199</v>
+        <v>245</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>615</v>
+        <v>851</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>1508</v>
+        <v>2268</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>3069</v>
+        <v>4582</v>
       </c>
       <c r="K8" s="23" t="n">
-        <v>5269</v>
+        <v>7493</v>
       </c>
       <c r="L8" s="23" t="n">
-        <v>7762</v>
+        <v>10705</v>
       </c>
       <c r="M8" s="23" t="n">
-        <v>10349</v>
+        <v>14013</v>
       </c>
       <c r="N8" s="23" t="n">
-        <v>10323</v>
+        <v>13892</v>
       </c>
       <c r="O8" s="23" t="n">
-        <v>10248</v>
+        <v>13748</v>
       </c>
       <c r="P8" s="23" t="n">
-        <v>10105</v>
+        <v>13557</v>
       </c>
       <c r="Q8" s="23" t="n">
-        <v>9897</v>
+        <v>13319</v>
       </c>
       <c r="R8" s="23" t="n">
-        <v>9680</v>
+        <v>13101</v>
       </c>
       <c r="S8" s="23" t="n">
-        <v>9495</v>
+        <v>13039</v>
       </c>
       <c r="T8" s="23" t="n">
-        <v>13396</v>
+        <v>20131</v>
       </c>
       <c r="U8" s="23" t="n">
-        <v>22486</v>
+        <v>38559</v>
       </c>
       <c r="V8" s="23" t="n">
-        <v>37122</v>
+        <v>68066</v>
       </c>
       <c r="W8" s="23" t="n">
-        <v>57549</v>
+        <v>106090</v>
       </c>
       <c r="X8" s="23" t="n">
-        <v>80868</v>
+        <v>149035</v>
       </c>
       <c r="Y8" s="23" t="n">
-        <v>104784</v>
+        <v>194044</v>
       </c>
     </row>
     <row r="10">
@@ -2988,73 +2988,73 @@
         <v>6</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>93</v>
+        <v>144</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>173</v>
+        <v>257</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>267</v>
+        <v>367</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>347</v>
+        <v>465</v>
       </c>
       <c r="L11" s="13" t="n">
-        <v>417</v>
+        <v>553</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>479</v>
+        <v>628</v>
       </c>
       <c r="N11" s="13" t="n">
-        <v>461</v>
+        <v>610</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>437</v>
+        <v>586</v>
       </c>
       <c r="P11" s="13" t="n">
-        <v>411</v>
+        <v>560</v>
       </c>
       <c r="Q11" s="13" t="n">
-        <v>395</v>
+        <v>549</v>
       </c>
       <c r="R11" s="13" t="n">
-        <v>390</v>
+        <v>571</v>
       </c>
       <c r="S11" s="13" t="n">
-        <v>408</v>
+        <v>651</v>
       </c>
       <c r="T11" s="13" t="n">
-        <v>766</v>
+        <v>1400</v>
       </c>
       <c r="U11" s="13" t="n">
-        <v>1257</v>
+        <v>2389</v>
       </c>
       <c r="V11" s="13" t="n">
-        <v>1885</v>
+        <v>3491</v>
       </c>
       <c r="W11" s="13" t="n">
-        <v>2491</v>
+        <v>4594</v>
       </c>
       <c r="X11" s="13" t="n">
-        <v>3039</v>
+        <v>5655</v>
       </c>
       <c r="Y11" s="13" t="n">
-        <v>3544</v>
+        <v>6599</v>
       </c>
     </row>
     <row r="12">
@@ -3079,10 +3079,10 @@
         <v>0</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>286</v>
+        <v>414</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>629</v>
+        <v>988</v>
       </c>
       <c r="I12" s="13" t="n">
         <v>0</v>
@@ -3115,10 +3115,10 @@
         <v>0</v>
       </c>
       <c r="S12" s="13" t="n">
-        <v>2119</v>
+        <v>3590</v>
       </c>
       <c r="T12" s="13" t="n">
-        <v>4398</v>
+        <v>8479</v>
       </c>
       <c r="U12" s="13" t="n">
         <v>0</v>
@@ -3146,73 +3146,73 @@
         <v>6</v>
       </c>
       <c r="C13" s="23" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E13" s="23" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G13" s="23" t="n">
-        <v>327</v>
+        <v>473</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>721</v>
+        <v>1133</v>
       </c>
       <c r="I13" s="23" t="n">
-        <v>173</v>
+        <v>257</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>267</v>
+        <v>367</v>
       </c>
       <c r="K13" s="23" t="n">
-        <v>347</v>
+        <v>465</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>417</v>
+        <v>553</v>
       </c>
       <c r="M13" s="23" t="n">
-        <v>479</v>
+        <v>628</v>
       </c>
       <c r="N13" s="23" t="n">
-        <v>461</v>
+        <v>610</v>
       </c>
       <c r="O13" s="23" t="n">
-        <v>437</v>
+        <v>586</v>
       </c>
       <c r="P13" s="23" t="n">
-        <v>411</v>
+        <v>560</v>
       </c>
       <c r="Q13" s="23" t="n">
-        <v>395</v>
+        <v>549</v>
       </c>
       <c r="R13" s="23" t="n">
-        <v>390</v>
+        <v>571</v>
       </c>
       <c r="S13" s="23" t="n">
-        <v>2527</v>
+        <v>4241</v>
       </c>
       <c r="T13" s="23" t="n">
-        <v>5163</v>
+        <v>9879</v>
       </c>
       <c r="U13" s="23" t="n">
-        <v>1257</v>
+        <v>2389</v>
       </c>
       <c r="V13" s="23" t="n">
-        <v>1885</v>
+        <v>3491</v>
       </c>
       <c r="W13" s="23" t="n">
-        <v>2491</v>
+        <v>4594</v>
       </c>
       <c r="X13" s="23" t="n">
-        <v>3039</v>
+        <v>5655</v>
       </c>
       <c r="Y13" s="23" t="n">
-        <v>3544</v>
+        <v>6599</v>
       </c>
     </row>
     <row r="15">
@@ -3307,22 +3307,22 @@
         <v>0</v>
       </c>
       <c r="T16" s="13" t="n">
-        <v>3525</v>
+        <v>6797</v>
       </c>
       <c r="U16" s="13" t="n">
-        <v>5726</v>
+        <v>11207</v>
       </c>
       <c r="V16" s="13" t="n">
-        <v>8283</v>
+        <v>15370</v>
       </c>
       <c r="W16" s="13" t="n">
-        <v>10220</v>
+        <v>18831</v>
       </c>
       <c r="X16" s="13" t="n">
-        <v>11580</v>
+        <v>21638</v>
       </c>
       <c r="Y16" s="13" t="n">
-        <v>12639</v>
+        <v>23597</v>
       </c>
     </row>
     <row r="18">
@@ -3366,73 +3366,73 @@
         <v>49</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>195</v>
+        <v>239</v>
       </c>
       <c r="F19" s="13" t="n">
-        <v>244</v>
+        <v>330</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>301</v>
+        <v>438</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>1629</v>
+        <v>2577</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>2874</v>
+        <v>4263</v>
       </c>
       <c r="J19" s="13" t="n">
-        <v>4111</v>
+        <v>5472</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>4770</v>
+        <v>6189</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>5094</v>
+        <v>6563</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>5210</v>
+        <v>6640</v>
       </c>
       <c r="N19" s="13" t="n">
-        <v>1974</v>
+        <v>2575</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>1819</v>
+        <v>2443</v>
       </c>
       <c r="P19" s="13" t="n">
-        <v>1658</v>
+        <v>2302</v>
       </c>
       <c r="Q19" s="13" t="n">
-        <v>1591</v>
+        <v>2284</v>
       </c>
       <c r="R19" s="13" t="n">
-        <v>1602</v>
+        <v>2530</v>
       </c>
       <c r="S19" s="13" t="n">
-        <v>1806</v>
+        <v>3222</v>
       </c>
       <c r="T19" s="13" t="n">
-        <v>10204</v>
+        <v>20429</v>
       </c>
       <c r="U19" s="13" t="n">
-        <v>16466</v>
+        <v>32949</v>
       </c>
       <c r="V19" s="13" t="n">
-        <v>23195</v>
+        <v>43141</v>
       </c>
       <c r="W19" s="13" t="n">
-        <v>27041</v>
+        <v>49805</v>
       </c>
       <c r="X19" s="13" t="n">
-        <v>28539</v>
+        <v>53597</v>
       </c>
       <c r="Y19" s="13" t="n">
-        <v>28943</v>
+        <v>54236</v>
       </c>
     </row>
     <row r="21">
@@ -3445,73 +3445,73 @@
         <v>55</v>
       </c>
       <c r="C21" s="15" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="D21" s="15" t="n">
-        <v>212</v>
+        <v>238</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>307</v>
+        <v>365</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>415</v>
+        <v>533</v>
       </c>
       <c r="G21" s="15" t="n">
-        <v>828</v>
+        <v>1156</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>2965</v>
+        <v>4560</v>
       </c>
       <c r="I21" s="15" t="n">
-        <v>4555</v>
+        <v>6788</v>
       </c>
       <c r="J21" s="15" t="n">
-        <v>7447</v>
+        <v>10421</v>
       </c>
       <c r="K21" s="15" t="n">
-        <v>10387</v>
+        <v>14147</v>
       </c>
       <c r="L21" s="15" t="n">
-        <v>13273</v>
+        <v>17820</v>
       </c>
       <c r="M21" s="15" t="n">
-        <v>16038</v>
+        <v>21281</v>
       </c>
       <c r="N21" s="15" t="n">
-        <v>12758</v>
+        <v>17077</v>
       </c>
       <c r="O21" s="15" t="n">
-        <v>12503</v>
+        <v>16777</v>
       </c>
       <c r="P21" s="15" t="n">
-        <v>12173</v>
+        <v>16420</v>
       </c>
       <c r="Q21" s="15" t="n">
-        <v>11884</v>
+        <v>16152</v>
       </c>
       <c r="R21" s="15" t="n">
-        <v>11672</v>
+        <v>16203</v>
       </c>
       <c r="S21" s="15" t="n">
-        <v>13829</v>
+        <v>20502</v>
       </c>
       <c r="T21" s="15" t="n">
-        <v>32288</v>
+        <v>57236</v>
       </c>
       <c r="U21" s="15" t="n">
-        <v>45935</v>
+        <v>85105</v>
       </c>
       <c r="V21" s="15" t="n">
-        <v>70485</v>
+        <v>130069</v>
       </c>
       <c r="W21" s="15" t="n">
-        <v>97301</v>
+        <v>179319</v>
       </c>
       <c r="X21" s="15" t="n">
-        <v>124027</v>
+        <v>229924</v>
       </c>
       <c r="Y21" s="15" t="n">
-        <v>149910</v>
+        <v>278476</v>
       </c>
       <c r="Z21" s="14" t="n"/>
     </row>
@@ -3525,73 +3525,73 @@
         <v>55</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>394</v>
+        <v>428</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>701</v>
+        <v>793</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>1116</v>
+        <v>1326</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>1944</v>
+        <v>2482</v>
       </c>
       <c r="H23" s="25" t="n">
-        <v>4909</v>
+        <v>7043</v>
       </c>
       <c r="I23" s="25" t="n">
-        <v>9464</v>
+        <v>13831</v>
       </c>
       <c r="J23" s="25" t="n">
-        <v>16911</v>
+        <v>24251</v>
       </c>
       <c r="K23" s="25" t="n">
-        <v>27298</v>
+        <v>38399</v>
       </c>
       <c r="L23" s="25" t="n">
-        <v>40571</v>
+        <v>56219</v>
       </c>
       <c r="M23" s="25" t="n">
-        <v>56609</v>
+        <v>77500</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>69368</v>
+        <v>94576</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>81871</v>
+        <v>111353</v>
       </c>
       <c r="P23" s="25" t="n">
-        <v>94044</v>
+        <v>127773</v>
       </c>
       <c r="Q23" s="25" t="n">
-        <v>105928</v>
+        <v>143925</v>
       </c>
       <c r="R23" s="25" t="n">
-        <v>117600</v>
+        <v>160128</v>
       </c>
       <c r="S23" s="25" t="n">
-        <v>131429</v>
+        <v>180630</v>
       </c>
       <c r="T23" s="25" t="n">
-        <v>163717</v>
+        <v>237867</v>
       </c>
       <c r="U23" s="25" t="n">
-        <v>209652</v>
+        <v>322972</v>
       </c>
       <c r="V23" s="25" t="n">
-        <v>280137</v>
+        <v>453040</v>
       </c>
       <c r="W23" s="25" t="n">
-        <v>377438</v>
+        <v>632360</v>
       </c>
       <c r="X23" s="25" t="n">
-        <v>501465</v>
+        <v>862284</v>
       </c>
       <c r="Y23" s="25" t="n">
-        <v>651375</v>
+        <v>1140760</v>
       </c>
     </row>
   </sheetData>
@@ -3821,7 +3821,7 @@
         <v>170</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D6" s="13" t="n">
         <v>171</v>
@@ -3830,64 +3830,64 @@
         <v>172</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>241</v>
+        <v>274</v>
       </c>
       <c r="L6" s="13" t="n">
-        <v>273</v>
+        <v>314</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>305</v>
+        <v>354</v>
       </c>
       <c r="N6" s="13" t="n">
-        <v>304</v>
+        <v>353</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>302</v>
+        <v>351</v>
       </c>
       <c r="P6" s="13" t="n">
-        <v>299</v>
+        <v>348</v>
       </c>
       <c r="Q6" s="13" t="n">
-        <v>297</v>
+        <v>345</v>
       </c>
       <c r="R6" s="13" t="n">
-        <v>294</v>
+        <v>345</v>
       </c>
       <c r="S6" s="13" t="n">
-        <v>294</v>
+        <v>351</v>
       </c>
       <c r="T6" s="13" t="n">
-        <v>363</v>
+        <v>484</v>
       </c>
       <c r="U6" s="13" t="n">
-        <v>498</v>
+        <v>757</v>
       </c>
       <c r="V6" s="13" t="n">
-        <v>703</v>
+        <v>1157</v>
       </c>
       <c r="W6" s="13" t="n">
-        <v>968</v>
+        <v>1649</v>
       </c>
       <c r="X6" s="13" t="n">
-        <v>1261</v>
+        <v>2192</v>
       </c>
       <c r="Y6" s="13" t="n">
-        <v>1557</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="8">
@@ -4425,67 +4425,67 @@
         <v>10</v>
       </c>
       <c r="E20" s="13" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>106</v>
+        <v>149</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>500</v>
+        <v>742</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>842</v>
+        <v>1194</v>
       </c>
       <c r="L20" s="13" t="n">
-        <v>1227</v>
+        <v>1689</v>
       </c>
       <c r="M20" s="13" t="n">
-        <v>1624</v>
+        <v>2196</v>
       </c>
       <c r="N20" s="13" t="n">
-        <v>1618</v>
+        <v>2175</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>1603</v>
+        <v>2150</v>
       </c>
       <c r="P20" s="13" t="n">
-        <v>1577</v>
+        <v>2118</v>
       </c>
       <c r="Q20" s="13" t="n">
-        <v>1544</v>
+        <v>2080</v>
       </c>
       <c r="R20" s="13" t="n">
-        <v>1510</v>
+        <v>2051</v>
       </c>
       <c r="S20" s="13" t="n">
-        <v>1486</v>
+        <v>2054</v>
       </c>
       <c r="T20" s="13" t="n">
-        <v>2124</v>
+        <v>3230</v>
       </c>
       <c r="U20" s="13" t="n">
-        <v>3561</v>
+        <v>6142</v>
       </c>
       <c r="V20" s="13" t="n">
-        <v>5851</v>
+        <v>10734</v>
       </c>
       <c r="W20" s="13" t="n">
-        <v>9006</v>
+        <v>16603</v>
       </c>
       <c r="X20" s="13" t="n">
-        <v>12586</v>
+        <v>23203</v>
       </c>
       <c r="Y20" s="13" t="n">
-        <v>16249</v>
+        <v>30096</v>
       </c>
     </row>
     <row r="21">
@@ -4510,10 +4510,10 @@
         <v>0</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="I21" s="13" t="n">
         <v>0</v>
@@ -4546,25 +4546,25 @@
         <v>0</v>
       </c>
       <c r="S21" s="13" t="n">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="T21" s="13" t="n">
-        <v>238</v>
+        <v>458</v>
       </c>
       <c r="U21" s="13" t="n">
-        <v>172</v>
+        <v>336</v>
       </c>
       <c r="V21" s="13" t="n">
-        <v>248</v>
+        <v>461</v>
       </c>
       <c r="W21" s="13" t="n">
-        <v>307</v>
+        <v>565</v>
       </c>
       <c r="X21" s="13" t="n">
-        <v>347</v>
+        <v>649</v>
       </c>
       <c r="Y21" s="13" t="n">
-        <v>379</v>
+        <v>708</v>
       </c>
     </row>
     <row r="22">
@@ -4583,67 +4583,67 @@
         <v>10</v>
       </c>
       <c r="E22" s="23" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G22" s="23" t="n">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="H22" s="23" t="n">
-        <v>125</v>
+        <v>179</v>
       </c>
       <c r="I22" s="23" t="n">
-        <v>252</v>
+        <v>379</v>
       </c>
       <c r="J22" s="23" t="n">
-        <v>500</v>
+        <v>742</v>
       </c>
       <c r="K22" s="23" t="n">
-        <v>842</v>
+        <v>1194</v>
       </c>
       <c r="L22" s="23" t="n">
-        <v>1227</v>
+        <v>1689</v>
       </c>
       <c r="M22" s="23" t="n">
-        <v>1624</v>
+        <v>2196</v>
       </c>
       <c r="N22" s="23" t="n">
-        <v>1618</v>
+        <v>2175</v>
       </c>
       <c r="O22" s="23" t="n">
-        <v>1603</v>
+        <v>2150</v>
       </c>
       <c r="P22" s="23" t="n">
-        <v>1577</v>
+        <v>2118</v>
       </c>
       <c r="Q22" s="23" t="n">
-        <v>1544</v>
+        <v>2080</v>
       </c>
       <c r="R22" s="23" t="n">
-        <v>1510</v>
+        <v>2051</v>
       </c>
       <c r="S22" s="23" t="n">
-        <v>1549</v>
+        <v>2161</v>
       </c>
       <c r="T22" s="23" t="n">
-        <v>2362</v>
+        <v>3688</v>
       </c>
       <c r="U22" s="23" t="n">
-        <v>3733</v>
+        <v>6478</v>
       </c>
       <c r="V22" s="23" t="n">
-        <v>6100</v>
+        <v>11195</v>
       </c>
       <c r="W22" s="23" t="n">
-        <v>9313</v>
+        <v>17168</v>
       </c>
       <c r="X22" s="23" t="n">
-        <v>12934</v>
+        <v>23853</v>
       </c>
       <c r="Y22" s="23" t="n">
-        <v>16628</v>
+        <v>30804</v>
       </c>
     </row>
     <row r="24">
@@ -4662,67 +4662,67 @@
         <v>761</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>5308</v>
+        <v>5311</v>
       </c>
       <c r="F24" s="15" t="n">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>4418</v>
+        <v>4432</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>2804</v>
+        <v>2862</v>
       </c>
       <c r="I24" s="15" t="n">
-        <v>8193</v>
+        <v>8332</v>
       </c>
       <c r="J24" s="15" t="n">
-        <v>3713</v>
+        <v>3978</v>
       </c>
       <c r="K24" s="15" t="n">
-        <v>4334</v>
+        <v>4717</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>9000</v>
+        <v>9502</v>
       </c>
       <c r="M24" s="15" t="n">
-        <v>10679</v>
+        <v>11300</v>
       </c>
       <c r="N24" s="15" t="n">
-        <v>7121</v>
+        <v>7728</v>
       </c>
       <c r="O24" s="15" t="n">
-        <v>6655</v>
+        <v>7251</v>
       </c>
       <c r="P24" s="15" t="n">
-        <v>12677</v>
+        <v>13265</v>
       </c>
       <c r="Q24" s="15" t="n">
-        <v>12690</v>
+        <v>13275</v>
       </c>
       <c r="R24" s="15" t="n">
-        <v>6705</v>
+        <v>7296</v>
       </c>
       <c r="S24" s="15" t="n">
-        <v>11793</v>
+        <v>12463</v>
       </c>
       <c r="T24" s="15" t="n">
-        <v>12225</v>
+        <v>13672</v>
       </c>
       <c r="U24" s="15" t="n">
-        <v>22731</v>
+        <v>25735</v>
       </c>
       <c r="V24" s="15" t="n">
-        <v>18302</v>
+        <v>23852</v>
       </c>
       <c r="W24" s="15" t="n">
-        <v>22781</v>
+        <v>31317</v>
       </c>
       <c r="X24" s="15" t="n">
-        <v>32695</v>
+        <v>44545</v>
       </c>
       <c r="Y24" s="15" t="n">
-        <v>38686</v>
+        <v>54054</v>
       </c>
       <c r="Z24" s="14" t="n"/>
     </row>
@@ -5257,73 +5257,73 @@
         <v>55</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>212</v>
+        <v>238</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>307</v>
+        <v>365</v>
       </c>
       <c r="F5" s="28" t="n">
-        <v>415</v>
+        <v>533</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>828</v>
+        <v>1156</v>
       </c>
       <c r="H5" s="28" t="n">
-        <v>2965</v>
+        <v>4560</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>4555</v>
+        <v>6788</v>
       </c>
       <c r="J5" s="28" t="n">
-        <v>7447</v>
+        <v>10421</v>
       </c>
       <c r="K5" s="28" t="n">
-        <v>10387</v>
+        <v>14147</v>
       </c>
       <c r="L5" s="28" t="n">
-        <v>13273</v>
+        <v>17820</v>
       </c>
       <c r="M5" s="28" t="n">
-        <v>16038</v>
+        <v>21281</v>
       </c>
       <c r="N5" s="28" t="n">
-        <v>12758</v>
+        <v>17077</v>
       </c>
       <c r="O5" s="28" t="n">
-        <v>12503</v>
+        <v>16777</v>
       </c>
       <c r="P5" s="28" t="n">
-        <v>12173</v>
+        <v>16420</v>
       </c>
       <c r="Q5" s="28" t="n">
-        <v>11884</v>
+        <v>16152</v>
       </c>
       <c r="R5" s="28" t="n">
-        <v>11672</v>
+        <v>16203</v>
       </c>
       <c r="S5" s="28" t="n">
-        <v>13829</v>
+        <v>20502</v>
       </c>
       <c r="T5" s="28" t="n">
-        <v>32288</v>
+        <v>57236</v>
       </c>
       <c r="U5" s="28" t="n">
-        <v>45935</v>
+        <v>85105</v>
       </c>
       <c r="V5" s="28" t="n">
-        <v>70485</v>
+        <v>130069</v>
       </c>
       <c r="W5" s="28" t="n">
-        <v>97301</v>
+        <v>179319</v>
       </c>
       <c r="X5" s="28" t="n">
-        <v>124027</v>
+        <v>229924</v>
       </c>
       <c r="Y5" s="28" t="n">
-        <v>149910</v>
+        <v>278476</v>
       </c>
     </row>
     <row r="6">
@@ -5342,67 +5342,67 @@
         <v>761</v>
       </c>
       <c r="E6" s="28" t="n">
-        <v>5308</v>
+        <v>5311</v>
       </c>
       <c r="F6" s="28" t="n">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="G6" s="28" t="n">
-        <v>4418</v>
+        <v>4432</v>
       </c>
       <c r="H6" s="28" t="n">
-        <v>2804</v>
+        <v>2862</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>8193</v>
+        <v>8332</v>
       </c>
       <c r="J6" s="28" t="n">
-        <v>3713</v>
+        <v>3978</v>
       </c>
       <c r="K6" s="28" t="n">
-        <v>4334</v>
+        <v>4717</v>
       </c>
       <c r="L6" s="28" t="n">
-        <v>9000</v>
+        <v>9502</v>
       </c>
       <c r="M6" s="28" t="n">
-        <v>10679</v>
+        <v>11300</v>
       </c>
       <c r="N6" s="28" t="n">
-        <v>7121</v>
+        <v>7728</v>
       </c>
       <c r="O6" s="28" t="n">
-        <v>6655</v>
+        <v>7251</v>
       </c>
       <c r="P6" s="28" t="n">
-        <v>12677</v>
+        <v>13265</v>
       </c>
       <c r="Q6" s="28" t="n">
-        <v>12690</v>
+        <v>13275</v>
       </c>
       <c r="R6" s="28" t="n">
-        <v>6705</v>
+        <v>7296</v>
       </c>
       <c r="S6" s="28" t="n">
-        <v>11793</v>
+        <v>12463</v>
       </c>
       <c r="T6" s="28" t="n">
-        <v>12225</v>
+        <v>13672</v>
       </c>
       <c r="U6" s="28" t="n">
-        <v>22731</v>
+        <v>25735</v>
       </c>
       <c r="V6" s="28" t="n">
-        <v>18302</v>
+        <v>23852</v>
       </c>
       <c r="W6" s="28" t="n">
-        <v>22781</v>
+        <v>31317</v>
       </c>
       <c r="X6" s="28" t="n">
-        <v>32695</v>
+        <v>44545</v>
       </c>
       <c r="Y6" s="28" t="n">
-        <v>38686</v>
+        <v>54054</v>
       </c>
     </row>
     <row r="8">
@@ -5415,73 +5415,73 @@
         <v>-1366</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>-587</v>
+        <v>-580</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>-549</v>
+        <v>-523</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>-5001</v>
+        <v>-4945</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>-443</v>
+        <v>-330</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>-3590</v>
+        <v>-3276</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>161</v>
+        <v>1698</v>
       </c>
       <c r="I8" s="15" t="n">
-        <v>-3638</v>
+        <v>-1544</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>3734</v>
+        <v>6443</v>
       </c>
       <c r="K8" s="15" t="n">
-        <v>6053</v>
+        <v>9430</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>4274</v>
+        <v>8318</v>
       </c>
       <c r="M8" s="15" t="n">
-        <v>5359</v>
+        <v>9980</v>
       </c>
       <c r="N8" s="15" t="n">
-        <v>5637</v>
+        <v>9349</v>
       </c>
       <c r="O8" s="15" t="n">
-        <v>5849</v>
+        <v>9526</v>
       </c>
       <c r="P8" s="15" t="n">
-        <v>-503</v>
+        <v>3154</v>
       </c>
       <c r="Q8" s="15" t="n">
-        <v>-807</v>
+        <v>2877</v>
       </c>
       <c r="R8" s="15" t="n">
-        <v>4967</v>
+        <v>8907</v>
       </c>
       <c r="S8" s="15" t="n">
-        <v>2035</v>
+        <v>8040</v>
       </c>
       <c r="T8" s="15" t="n">
-        <v>20063</v>
+        <v>43564</v>
       </c>
       <c r="U8" s="15" t="n">
-        <v>23204</v>
+        <v>59370</v>
       </c>
       <c r="V8" s="15" t="n">
-        <v>52183</v>
+        <v>106217</v>
       </c>
       <c r="W8" s="15" t="n">
-        <v>74520</v>
+        <v>148003</v>
       </c>
       <c r="X8" s="15" t="n">
-        <v>91332</v>
+        <v>185380</v>
       </c>
       <c r="Y8" s="15" t="n">
-        <v>111225</v>
+        <v>224422</v>
       </c>
       <c r="Z8" s="14" t="n"/>
     </row>
@@ -5495,73 +5495,73 @@
         <v>-24.87</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>-4.62</v>
+        <v>-4.31</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>-2.59</v>
+        <v>-2.19</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>-16.29</v>
+        <v>-13.53</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>-1.07</v>
+        <v>-0.62</v>
       </c>
       <c r="G9" s="29" t="n">
-        <v>-4.34</v>
+        <v>-2.83</v>
       </c>
       <c r="H9" s="29" t="n">
-        <v>0.05</v>
+        <v>0.37</v>
       </c>
       <c r="I9" s="29" t="n">
-        <v>-0.8</v>
+        <v>-0.23</v>
       </c>
       <c r="J9" s="29" t="n">
-        <v>0.5</v>
+        <v>0.62</v>
       </c>
       <c r="K9" s="29" t="n">
-        <v>0.58</v>
+        <v>0.67</v>
       </c>
       <c r="L9" s="29" t="n">
-        <v>0.32</v>
+        <v>0.47</v>
       </c>
       <c r="M9" s="29" t="n">
-        <v>0.33</v>
+        <v>0.47</v>
       </c>
       <c r="N9" s="29" t="n">
-        <v>0.44</v>
+        <v>0.55</v>
       </c>
       <c r="O9" s="29" t="n">
-        <v>0.47</v>
+        <v>0.57</v>
       </c>
       <c r="P9" s="29" t="n">
-        <v>-0.04</v>
+        <v>0.19</v>
       </c>
       <c r="Q9" s="29" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="R9" s="29" t="n">
-        <v>0.43</v>
+        <v>0.55</v>
       </c>
       <c r="S9" s="29" t="n">
-        <v>0.15</v>
+        <v>0.39</v>
       </c>
       <c r="T9" s="29" t="n">
-        <v>0.62</v>
+        <v>0.76</v>
       </c>
       <c r="U9" s="29" t="n">
-        <v>0.51</v>
+        <v>0.7</v>
       </c>
       <c r="V9" s="29" t="n">
-        <v>0.74</v>
+        <v>0.82</v>
       </c>
       <c r="W9" s="29" t="n">
-        <v>0.77</v>
+        <v>0.83</v>
       </c>
       <c r="X9" s="29" t="n">
-        <v>0.74</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y9" s="29" t="n">
-        <v>0.74</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -5574,73 +5574,73 @@
         <v>55</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>394</v>
+        <v>428</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>701</v>
+        <v>793</v>
       </c>
       <c r="F11" s="28" t="n">
-        <v>1116</v>
+        <v>1326</v>
       </c>
       <c r="G11" s="28" t="n">
-        <v>1944</v>
+        <v>2482</v>
       </c>
       <c r="H11" s="28" t="n">
-        <v>4909</v>
+        <v>7043</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>9464</v>
+        <v>13831</v>
       </c>
       <c r="J11" s="28" t="n">
-        <v>16911</v>
+        <v>24251</v>
       </c>
       <c r="K11" s="28" t="n">
-        <v>27298</v>
+        <v>38399</v>
       </c>
       <c r="L11" s="28" t="n">
-        <v>40571</v>
+        <v>56219</v>
       </c>
       <c r="M11" s="28" t="n">
-        <v>56609</v>
+        <v>77500</v>
       </c>
       <c r="N11" s="28" t="n">
-        <v>69368</v>
+        <v>94576</v>
       </c>
       <c r="O11" s="28" t="n">
-        <v>81871</v>
+        <v>111353</v>
       </c>
       <c r="P11" s="28" t="n">
-        <v>94044</v>
+        <v>127773</v>
       </c>
       <c r="Q11" s="28" t="n">
-        <v>105928</v>
+        <v>143925</v>
       </c>
       <c r="R11" s="28" t="n">
-        <v>117600</v>
+        <v>160128</v>
       </c>
       <c r="S11" s="28" t="n">
-        <v>131429</v>
+        <v>180630</v>
       </c>
       <c r="T11" s="28" t="n">
-        <v>163717</v>
+        <v>237867</v>
       </c>
       <c r="U11" s="28" t="n">
-        <v>209652</v>
+        <v>322972</v>
       </c>
       <c r="V11" s="28" t="n">
-        <v>280137</v>
+        <v>453040</v>
       </c>
       <c r="W11" s="28" t="n">
-        <v>377438</v>
+        <v>632360</v>
       </c>
       <c r="X11" s="28" t="n">
-        <v>501465</v>
+        <v>862284</v>
       </c>
       <c r="Y11" s="28" t="n">
-        <v>651375</v>
+        <v>1140760</v>
       </c>
     </row>
     <row r="12">
@@ -5653,73 +5653,73 @@
         <v>-1366</v>
       </c>
       <c r="C12" s="30" t="n">
-        <v>-1953</v>
+        <v>-1946</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>-2502</v>
+        <v>-2469</v>
       </c>
       <c r="E12" s="30" t="n">
-        <v>-7504</v>
+        <v>-7415</v>
       </c>
       <c r="F12" s="30" t="n">
-        <v>-7947</v>
+        <v>-7745</v>
       </c>
       <c r="G12" s="30" t="n">
-        <v>-11537</v>
+        <v>-11021</v>
       </c>
       <c r="H12" s="30" t="n">
-        <v>-11376</v>
+        <v>-9323</v>
       </c>
       <c r="I12" s="30" t="n">
-        <v>-15014</v>
+        <v>-10867</v>
       </c>
       <c r="J12" s="30" t="n">
-        <v>-11280</v>
-      </c>
-      <c r="K12" s="30" t="n">
-        <v>-5227</v>
-      </c>
-      <c r="L12" s="30" t="n">
-        <v>-953</v>
+        <v>-4424</v>
+      </c>
+      <c r="K12" s="31" t="n">
+        <v>5006</v>
+      </c>
+      <c r="L12" s="31" t="n">
+        <v>13323</v>
       </c>
       <c r="M12" s="31" t="n">
-        <v>4406</v>
+        <v>23304</v>
       </c>
       <c r="N12" s="31" t="n">
-        <v>10043</v>
+        <v>32652</v>
       </c>
       <c r="O12" s="31" t="n">
-        <v>15891</v>
+        <v>42179</v>
       </c>
       <c r="P12" s="31" t="n">
-        <v>15388</v>
+        <v>45333</v>
       </c>
       <c r="Q12" s="31" t="n">
-        <v>14582</v>
+        <v>48210</v>
       </c>
       <c r="R12" s="31" t="n">
-        <v>19549</v>
+        <v>57117</v>
       </c>
       <c r="S12" s="31" t="n">
-        <v>21584</v>
+        <v>65157</v>
       </c>
       <c r="T12" s="31" t="n">
-        <v>41647</v>
+        <v>108721</v>
       </c>
       <c r="U12" s="31" t="n">
-        <v>64851</v>
+        <v>168091</v>
       </c>
       <c r="V12" s="31" t="n">
-        <v>117033</v>
+        <v>274308</v>
       </c>
       <c r="W12" s="31" t="n">
-        <v>191553</v>
+        <v>422310</v>
       </c>
       <c r="X12" s="31" t="n">
-        <v>282885</v>
+        <v>607690</v>
       </c>
       <c r="Y12" s="31" t="n">
-        <v>394110</v>
+        <v>832112</v>
       </c>
     </row>
     <row r="14">
@@ -5732,73 +5732,73 @@
         <v>150</v>
       </c>
       <c r="C14" s="28" t="n">
-        <v>308</v>
+        <v>328</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>461</v>
+        <v>528</v>
       </c>
       <c r="E14" s="28" t="n">
-        <v>613</v>
+        <v>749</v>
       </c>
       <c r="F14" s="28" t="n">
-        <v>771</v>
+        <v>1038</v>
       </c>
       <c r="G14" s="28" t="n">
-        <v>956</v>
+        <v>1383</v>
       </c>
       <c r="H14" s="28" t="n">
-        <v>2100</v>
+        <v>3301</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>3776</v>
+        <v>5606</v>
       </c>
       <c r="J14" s="28" t="n">
-        <v>5555</v>
+        <v>7479</v>
       </c>
       <c r="K14" s="28" t="n">
-        <v>6734</v>
+        <v>8847</v>
       </c>
       <c r="L14" s="28" t="n">
-        <v>7550</v>
+        <v>9845</v>
       </c>
       <c r="M14" s="28" t="n">
-        <v>8127</v>
+        <v>10496</v>
       </c>
       <c r="N14" s="28" t="n">
-        <v>7773</v>
+        <v>10210</v>
       </c>
       <c r="O14" s="28" t="n">
-        <v>7273</v>
+        <v>9767</v>
       </c>
       <c r="P14" s="28" t="n">
-        <v>6747</v>
+        <v>9289</v>
       </c>
       <c r="Q14" s="28" t="n">
-        <v>6499</v>
+        <v>9182</v>
       </c>
       <c r="R14" s="28" t="n">
-        <v>6487</v>
+        <v>9890</v>
       </c>
       <c r="S14" s="28" t="n">
-        <v>7076</v>
+        <v>11990</v>
       </c>
       <c r="T14" s="28" t="n">
-        <v>14688</v>
+        <v>28320</v>
       </c>
       <c r="U14" s="28" t="n">
-        <v>23858</v>
+        <v>46698</v>
       </c>
       <c r="V14" s="28" t="n">
-        <v>34512</v>
+        <v>64043</v>
       </c>
       <c r="W14" s="28" t="n">
-        <v>42583</v>
+        <v>78461</v>
       </c>
       <c r="X14" s="28" t="n">
-        <v>48249</v>
+        <v>90159</v>
       </c>
       <c r="Y14" s="28" t="n">
-        <v>52663</v>
+        <v>98320</v>
       </c>
     </row>
     <row r="15">
@@ -5817,67 +5817,67 @@
         <v>8</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F15" s="28" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G15" s="28" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H15" s="28" t="n">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>254</v>
+        <v>383</v>
       </c>
       <c r="J15" s="28" t="n">
-        <v>517</v>
+        <v>773</v>
       </c>
       <c r="K15" s="28" t="n">
-        <v>888</v>
+        <v>1263</v>
       </c>
       <c r="L15" s="28" t="n">
-        <v>1308</v>
+        <v>1803</v>
       </c>
       <c r="M15" s="28" t="n">
-        <v>1742</v>
+        <v>2359</v>
       </c>
       <c r="N15" s="28" t="n">
-        <v>1725</v>
+        <v>2321</v>
       </c>
       <c r="O15" s="28" t="n">
-        <v>1701</v>
+        <v>2282</v>
       </c>
       <c r="P15" s="28" t="n">
-        <v>1667</v>
+        <v>2237</v>
       </c>
       <c r="Q15" s="28" t="n">
-        <v>1624</v>
+        <v>2185</v>
       </c>
       <c r="R15" s="28" t="n">
-        <v>1580</v>
+        <v>2138</v>
       </c>
       <c r="S15" s="28" t="n">
-        <v>1542</v>
+        <v>2118</v>
       </c>
       <c r="T15" s="28" t="n">
-        <v>2183</v>
+        <v>3284</v>
       </c>
       <c r="U15" s="28" t="n">
-        <v>3679</v>
+        <v>6319</v>
       </c>
       <c r="V15" s="28" t="n">
-        <v>6087</v>
+        <v>11175</v>
       </c>
       <c r="W15" s="28" t="n">
-        <v>9445</v>
+        <v>17426</v>
       </c>
       <c r="X15" s="28" t="n">
-        <v>13274</v>
+        <v>24477</v>
       </c>
       <c r="Y15" s="28" t="n">
-        <v>17194</v>
+        <v>31855</v>
       </c>
     </row>
     <row r="16">
@@ -5893,70 +5893,70 @@
         <v>0.41</v>
       </c>
       <c r="D16" s="32" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="E16" s="32" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="F16" s="32" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="G16" s="32" t="n">
-        <v>0.87</v>
+        <v>0.84</v>
       </c>
       <c r="H16" s="32" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="I16" s="32" t="n">
         <v>1.21</v>
       </c>
       <c r="J16" s="32" t="n">
-        <v>1.34</v>
+        <v>1.39</v>
       </c>
       <c r="K16" s="32" t="n">
-        <v>1.54</v>
+        <v>1.6</v>
       </c>
       <c r="L16" s="32" t="n">
-        <v>1.76</v>
+        <v>1.81</v>
       </c>
       <c r="M16" s="32" t="n">
-        <v>1.97</v>
+        <v>2.03</v>
       </c>
       <c r="N16" s="32" t="n">
-        <v>1.64</v>
+        <v>1.67</v>
       </c>
       <c r="O16" s="32" t="n">
         <v>1.72</v>
       </c>
       <c r="P16" s="32" t="n">
-        <v>1.8</v>
+        <v>1.77</v>
       </c>
       <c r="Q16" s="32" t="n">
-        <v>1.83</v>
+        <v>1.76</v>
       </c>
       <c r="R16" s="32" t="n">
-        <v>1.8</v>
+        <v>1.64</v>
       </c>
       <c r="S16" s="32" t="n">
-        <v>1.95</v>
+        <v>1.71</v>
       </c>
       <c r="T16" s="32" t="n">
-        <v>2.2</v>
+        <v>2.02</v>
       </c>
       <c r="U16" s="32" t="n">
-        <v>1.93</v>
+        <v>1.82</v>
       </c>
       <c r="V16" s="32" t="n">
-        <v>2.04</v>
+        <v>2.03</v>
       </c>
       <c r="W16" s="32" t="n">
-        <v>2.28</v>
+        <v>2.29</v>
       </c>
       <c r="X16" s="32" t="n">
-        <v>2.57</v>
+        <v>2.55</v>
       </c>
       <c r="Y16" s="32" t="n">
-        <v>2.85</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="17">
@@ -5969,73 +5969,73 @@
         <v>9.470000000000001</v>
       </c>
       <c r="C17" s="32" t="n">
-        <v>2.32</v>
+        <v>2.18</v>
       </c>
       <c r="D17" s="32" t="n">
-        <v>1.65</v>
+        <v>1.44</v>
       </c>
       <c r="E17" s="32" t="n">
-        <v>8.67</v>
+        <v>7.09</v>
       </c>
       <c r="F17" s="32" t="n">
-        <v>1.11</v>
+        <v>0.83</v>
       </c>
       <c r="G17" s="32" t="n">
-        <v>4.62</v>
+        <v>3.2</v>
       </c>
       <c r="H17" s="32" t="n">
-        <v>1.34</v>
+        <v>0.87</v>
       </c>
       <c r="I17" s="32" t="n">
-        <v>2.17</v>
+        <v>1.49</v>
       </c>
       <c r="J17" s="32" t="n">
-        <v>0.67</v>
+        <v>0.53</v>
       </c>
       <c r="K17" s="32" t="n">
-        <v>0.64</v>
+        <v>0.53</v>
       </c>
       <c r="L17" s="32" t="n">
-        <v>1.19</v>
+        <v>0.97</v>
       </c>
       <c r="M17" s="32" t="n">
-        <v>1.31</v>
+        <v>1.08</v>
       </c>
       <c r="N17" s="32" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="O17" s="32" t="n">
-        <v>0.92</v>
+        <v>0.74</v>
       </c>
       <c r="P17" s="32" t="n">
-        <v>1.88</v>
+        <v>1.43</v>
       </c>
       <c r="Q17" s="32" t="n">
-        <v>1.95</v>
+        <v>1.45</v>
       </c>
       <c r="R17" s="32" t="n">
-        <v>1.03</v>
+        <v>0.74</v>
       </c>
       <c r="S17" s="32" t="n">
-        <v>1.67</v>
+        <v>1.04</v>
       </c>
       <c r="T17" s="32" t="n">
-        <v>0.83</v>
+        <v>0.48</v>
       </c>
       <c r="U17" s="32" t="n">
-        <v>0.95</v>
+        <v>0.55</v>
       </c>
       <c r="V17" s="32" t="n">
-        <v>0.53</v>
+        <v>0.37</v>
       </c>
       <c r="W17" s="32" t="n">
-        <v>0.53</v>
+        <v>0.4</v>
       </c>
       <c r="X17" s="32" t="n">
-        <v>0.68</v>
+        <v>0.49</v>
       </c>
       <c r="Y17" s="32" t="n">
-        <v>0.73</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="18">
@@ -6048,73 +6048,73 @@
         <v>0.04</v>
       </c>
       <c r="C18" s="33" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="D18" s="33" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F18" s="33" t="n">
-        <v>0.48</v>
+        <v>0.62</v>
       </c>
       <c r="G18" s="33" t="n">
-        <v>0.19</v>
+        <v>0.26</v>
       </c>
       <c r="H18" s="33" t="n">
-        <v>1.06</v>
+        <v>1.59</v>
       </c>
       <c r="I18" s="33" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="J18" s="33" t="n">
-        <v>2.01</v>
+        <v>2.62</v>
       </c>
       <c r="K18" s="33" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="L18" s="33" t="n">
-        <v>1.47</v>
+        <v>1.88</v>
       </c>
       <c r="M18" s="33" t="n">
-        <v>1.5</v>
+        <v>1.88</v>
       </c>
       <c r="N18" s="33" t="n">
-        <v>1.79</v>
+        <v>2.21</v>
       </c>
       <c r="O18" s="33" t="n">
-        <v>1.88</v>
+        <v>2.31</v>
       </c>
       <c r="P18" s="33" t="n">
-        <v>0.96</v>
+        <v>1.24</v>
       </c>
       <c r="Q18" s="33" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.22</v>
       </c>
       <c r="R18" s="33" t="n">
-        <v>1.74</v>
+        <v>2.22</v>
       </c>
       <c r="S18" s="33" t="n">
-        <v>1.17</v>
+        <v>1.65</v>
       </c>
       <c r="T18" s="33" t="n">
-        <v>2.64</v>
+        <v>4.19</v>
       </c>
       <c r="U18" s="33" t="n">
-        <v>2.02</v>
+        <v>3.31</v>
       </c>
       <c r="V18" s="33" t="n">
-        <v>3.85</v>
+        <v>5.45</v>
       </c>
       <c r="W18" s="33" t="n">
-        <v>4.27</v>
+        <v>5.73</v>
       </c>
       <c r="X18" s="33" t="n">
-        <v>3.79</v>
+        <v>5.16</v>
       </c>
       <c r="Y18" s="33" t="n">
-        <v>3.88</v>
+        <v>5.15</v>
       </c>
     </row>
   </sheetData>
@@ -6184,10 +6184,10 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>8127</v>
+        <v>10496</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>52663</v>
+        <v>98320</v>
       </c>
     </row>
     <row r="6">
@@ -6197,10 +6197,10 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1411</v>
+        <v>1910</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>13396</v>
+        <v>24837</v>
       </c>
     </row>
     <row r="7">
@@ -6210,10 +6210,10 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>331</v>
+        <v>449</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>3798</v>
+        <v>7018</v>
       </c>
     </row>
     <row r="8">
@@ -6224,12 +6224,12 @@
       </c>
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="C8" s="34" t="inlineStr">
         <is>
-          <t>32.6%</t>
+          <t>32.4%</t>
         </is>
       </c>
     </row>
@@ -6247,13 +6247,13 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>29055.83778648977</v>
+        <v>40473.44582288782</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>375953.5188121126</v>
+        <v>656580.5629780137</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>11.93900115958527</v>
+        <v>15.22250217713649</v>
       </c>
     </row>
     <row r="12">
@@ -6263,13 +6263,13 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>2828.505765368695</v>
+        <v>3990.98824231727</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>22000.1772947998</v>
+        <v>39726.70780446646</v>
       </c>
       <c r="D12" s="29" t="n">
-        <v>6.778021018787664</v>
+        <v>8.95410294203225</v>
       </c>
     </row>
     <row r="13">
@@ -6282,7 +6282,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>51972.68030594899</v>
+        <v>97440.56159601365</v>
       </c>
       <c r="D13" s="35" t="inlineStr">
         <is>
@@ -6297,13 +6297,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>24725.06475290264</v>
+        <v>33035.09568619764</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>144839.4747467341</v>
+        <v>269512.4569919152</v>
       </c>
       <c r="D14" s="29" t="n">
-        <v>4.858001837173366</v>
+        <v>7.158367681208802</v>
       </c>
     </row>
     <row r="15">
@@ -6313,13 +6313,13 @@
         </is>
       </c>
       <c r="B15" s="23" t="n">
-        <v>56609.40830476111</v>
+        <v>77499.52975140273</v>
       </c>
       <c r="C15" s="23" t="n">
-        <v>594765.8511595955</v>
+        <v>1063260.289370409</v>
       </c>
       <c r="D15" s="29" t="n">
-        <v>9.506484151143706</v>
+        <v>12.71957085134654</v>
       </c>
     </row>
     <row r="17">
@@ -6336,10 +6336,10 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>2430.414766542152</v>
+        <v>2594.255308637736</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>7141.681909839889</v>
+        <v>11081.30988538878</v>
       </c>
     </row>
     <row r="19">
@@ -6388,10 +6388,10 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>4672.849637999113</v>
+        <v>6501.377667966505</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>60470.29998735372</v>
+        <v>105921.052784682</v>
       </c>
     </row>
     <row r="23">
@@ -6401,13 +6401,13 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>52203.26440454126</v>
+        <v>54195.63297660425</v>
       </c>
       <c r="C23" s="23" t="n">
-        <v>205061.9818971936</v>
+        <v>254452.3626700708</v>
       </c>
       <c r="D23" s="29" t="n">
-        <v>2.928144805430116</v>
+        <v>3.695071331299249</v>
       </c>
     </row>
     <row r="25">
@@ -6424,10 +6424,10 @@
         </is>
       </c>
       <c r="B26" s="36" t="n">
-        <v>4406.143900219853</v>
+        <v>23303.89677479849</v>
       </c>
       <c r="C26" s="36" t="n">
-        <v>389703.8692624019</v>
+        <v>808807.9267003383</v>
       </c>
     </row>
     <row r="27">
@@ -6437,10 +6437,10 @@
         </is>
       </c>
       <c r="B27" s="16" t="n">
-        <v>0.07783412743865892</v>
+        <v>0.3006972668034374</v>
       </c>
       <c r="C27" s="16" t="n">
-        <v>0.655222334138063</v>
+        <v>0.7606866679646803</v>
       </c>
     </row>
   </sheetData>
@@ -6525,16 +6525,16 @@
         </is>
       </c>
       <c r="B6" s="37" t="n">
-        <v>737</v>
+        <v>1376</v>
       </c>
       <c r="C6" s="37" t="n">
-        <v>184</v>
+        <v>344</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>66245</v>
+        <v>123677</v>
       </c>
       <c r="E6" s="38" t="n">
-        <v>-0.8237950761875651</v>
+        <v>-0.8116348214251773</v>
       </c>
     </row>
     <row r="7">
@@ -6544,16 +6544,16 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
-        <v>1290</v>
+        <v>2409</v>
       </c>
       <c r="C7" s="37" t="n">
-        <v>323</v>
+        <v>602</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>115929</v>
+        <v>216435</v>
       </c>
       <c r="E7" s="38" t="n">
-        <v>-0.6916413833282389</v>
+        <v>-0.6703609374940602</v>
       </c>
     </row>
     <row r="8">
@@ -6563,16 +6563,16 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
-        <v>2028</v>
+        <v>3785</v>
       </c>
       <c r="C8" s="39" t="n">
-        <v>507</v>
+        <v>946</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>182173</v>
+        <v>340112</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>-0.515436459515804</v>
+        <v>-0.4819957589192374</v>
       </c>
     </row>
     <row r="9">
@@ -6582,16 +6582,16 @@
         </is>
       </c>
       <c r="B9" s="37" t="n">
-        <v>2949</v>
+        <v>5506</v>
       </c>
       <c r="C9" s="37" t="n">
-        <v>737</v>
+        <v>1376</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>264979</v>
+        <v>494708</v>
       </c>
       <c r="E9" s="38" t="n">
-        <v>-0.2951803047502605</v>
+        <v>-0.2465392857007092</v>
       </c>
     </row>
     <row r="10">
@@ -6601,16 +6601,16 @@
         </is>
       </c>
       <c r="B10" s="37" t="n">
-        <v>3686</v>
+        <v>6882</v>
       </c>
       <c r="C10" s="37" t="n">
-        <v>922</v>
+        <v>1721</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>331224</v>
+        <v>618385</v>
       </c>
       <c r="E10" s="38" t="n">
-        <v>-0.1189753809378252</v>
+        <v>-0.05817410712588633</v>
       </c>
     </row>
     <row r="13">
@@ -6813,13 +6813,13 @@
         </is>
       </c>
       <c r="B24" s="28" t="n">
-        <v>4063</v>
+        <v>5248</v>
       </c>
       <c r="C24" s="28" t="n">
-        <v>26332</v>
+        <v>49160</v>
       </c>
       <c r="D24" s="28" t="n">
-        <v>267645</v>
+        <v>478467</v>
       </c>
       <c r="E24" s="37" t="inlineStr">
         <is>
@@ -6834,17 +6834,17 @@
         </is>
       </c>
       <c r="B25" s="25" t="n">
-        <v>8127</v>
+        <v>10496</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>52663</v>
+        <v>98320</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>594766</v>
+        <v>1063260</v>
       </c>
       <c r="E25" s="39" t="inlineStr">
         <is>
-          <t>Month 12</t>
+          <t>Month 10</t>
         </is>
       </c>
     </row>
@@ -6855,13 +6855,13 @@
         </is>
       </c>
       <c r="B26" s="28" t="n">
-        <v>16254</v>
+        <v>20992</v>
       </c>
       <c r="C26" s="28" t="n">
-        <v>131658</v>
+        <v>245800</v>
       </c>
       <c r="D26" s="28" t="n">
-        <v>1665344</v>
+        <v>2977129</v>
       </c>
       <c r="E26" s="37" t="inlineStr">
         <is>
@@ -6876,13 +6876,13 @@
         </is>
       </c>
       <c r="B27" s="28" t="n">
-        <v>40635</v>
+        <v>52480</v>
       </c>
       <c r="C27" s="28" t="n">
-        <v>421304</v>
+        <v>786561</v>
       </c>
       <c r="D27" s="28" t="n">
-        <v>5352893</v>
+        <v>9569343</v>
       </c>
       <c r="E27" s="37" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix DFS regulatory to Canadian jurisdiction — not US state-by-state
Canada-based company operating under Canadian law:

- Criminal Code s.206 skill contest exemption (federal)
- Ontario iGaming registration (AGCO/iGO): $2,000/mo amortized
- Gaming compliance counsel (FINTRAC AML): $2,500/mo
- Insurance / bonding (E&O, player fund segregation): $800/mo
- Provincial registration fees (AB/BC/QC nominal): $500/mo
- Total at 100K users: ~$5,800/mo (vs $13,500/mo US model)

Canadian DFS regulatory is dramatically cheaper than US — no $50K
per-state licensing. Main costs are Ontario iGaming registration,
FINTRAC anti-money-laundering compliance, and gaming counsel.

Sources updated with Canadian-specific citations (Criminal Code,
iGaming Ontario, AGCO, FINTRAC).

https://claude.ai/code/session_01DWcMBbfjeLfgrVr7i298sA
</commit_message>
<xml_diff>
--- a/docs/Citrus_Business_Model.xlsx
+++ b/docs/Citrus_Business_Model.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1797,7 +1797,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DFS REGULATORY (post-100K users)</t>
+          <t>DFS REGULATORY — CANADA (post-100K users)</t>
         </is>
       </c>
     </row>
@@ -1824,11 +1824,11 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>State Licensing (amortized)</t>
+          <t>Ontario iGaming Registration</t>
         </is>
       </c>
       <c r="B86" s="8" t="n">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
@@ -1837,18 +1837,18 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10-15 states @ $5K-50K each / 12mo</t>
+          <t>iGaming Ontario reg + annual fees amortized</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Compliance &amp; Legal Counsel</t>
+          <t>Gaming Compliance Counsel</t>
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
@@ -1857,18 +1857,18 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Ongoing regulatory, audits</t>
+          <t>Canadian gaming law, FINTRAC AML</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Regulatory Insurance / Bond</t>
+          <t>Insurance / Bonding</t>
         </is>
       </c>
       <c r="B88" s="8" t="n">
-        <v>1500</v>
+        <v>800</v>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
@@ -1877,48 +1877,48 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Surety bonds, E&amp;O insurance</t>
+          <t>E&amp;O, player fund segregation</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Provincial Registration Fees</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="n">
+        <v>500</v>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>USD/mo</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>AB/BC/QC nominal fees amortized</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>USER GROWTH / ACQUISITION (Monthly New Users)</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  New Users — Apr-26</t>
-        </is>
-      </c>
-      <c r="B91" s="8" t="n">
-        <v>150</v>
-      </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>users</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Monthly new user target</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — May-26</t>
+          <t xml:space="preserve">  New Users — Apr-26</t>
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
@@ -1934,11 +1934,11 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jun-26</t>
+          <t xml:space="preserve">  New Users — May-26</t>
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
@@ -1954,11 +1954,11 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jul-26</t>
+          <t xml:space="preserve">  New Users — Jun-26</t>
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
@@ -1974,11 +1974,11 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Aug-26</t>
+          <t xml:space="preserve">  New Users — Jul-26</t>
         </is>
       </c>
       <c r="B95" s="8" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
@@ -1994,11 +1994,11 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Sep-26</t>
+          <t xml:space="preserve">  New Users — Aug-26</t>
         </is>
       </c>
       <c r="B96" s="8" t="n">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
@@ -2014,11 +2014,11 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Oct-26</t>
+          <t xml:space="preserve">  New Users — Sep-26</t>
         </is>
       </c>
       <c r="B97" s="8" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
@@ -2034,11 +2034,11 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Nov-26</t>
+          <t xml:space="preserve">  New Users — Oct-26</t>
         </is>
       </c>
       <c r="B98" s="8" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
@@ -2054,11 +2054,11 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Dec-26</t>
+          <t xml:space="preserve">  New Users — Nov-26</t>
         </is>
       </c>
       <c r="B99" s="8" t="n">
-        <v>2200</v>
+        <v>2500</v>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
@@ -2074,11 +2074,11 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jan-27</t>
+          <t xml:space="preserve">  New Users — Dec-26</t>
         </is>
       </c>
       <c r="B100" s="8" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
@@ -2094,11 +2094,11 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Feb-27</t>
+          <t xml:space="preserve">  New Users — Jan-27</t>
         </is>
       </c>
       <c r="B101" s="8" t="n">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
@@ -2114,11 +2114,11 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Mar-27</t>
+          <t xml:space="preserve">  New Users — Feb-27</t>
         </is>
       </c>
       <c r="B102" s="8" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
@@ -2134,7 +2134,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Apr-27</t>
+          <t xml:space="preserve">  New Users — Mar-27</t>
         </is>
       </c>
       <c r="B103" s="8" t="n">
@@ -2154,11 +2154,11 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — May-27</t>
+          <t xml:space="preserve">  New Users — Apr-27</t>
         </is>
       </c>
       <c r="B104" s="8" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
@@ -2174,11 +2174,11 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jun-27</t>
+          <t xml:space="preserve">  New Users — May-27</t>
         </is>
       </c>
       <c r="B105" s="8" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
@@ -2194,11 +2194,11 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jul-27</t>
+          <t xml:space="preserve">  New Users — Jun-27</t>
         </is>
       </c>
       <c r="B106" s="8" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
@@ -2214,11 +2214,11 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Aug-27</t>
+          <t xml:space="preserve">  New Users — Jul-27</t>
         </is>
       </c>
       <c r="B107" s="8" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
@@ -2234,11 +2234,11 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Sep-27</t>
+          <t xml:space="preserve">  New Users — Aug-27</t>
         </is>
       </c>
       <c r="B108" s="8" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
@@ -2254,11 +2254,11 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Oct-27</t>
+          <t xml:space="preserve">  New Users — Sep-27</t>
         </is>
       </c>
       <c r="B109" s="8" t="n">
-        <v>17000</v>
+        <v>3500</v>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
@@ -2274,11 +2274,11 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Nov-27</t>
+          <t xml:space="preserve">  New Users — Oct-27</t>
         </is>
       </c>
       <c r="B110" s="8" t="n">
-        <v>20000</v>
+        <v>17000</v>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
@@ -2294,7 +2294,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Dec-27</t>
+          <t xml:space="preserve">  New Users — Nov-27</t>
         </is>
       </c>
       <c r="B111" s="8" t="n">
@@ -2314,11 +2314,11 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jan-28</t>
+          <t xml:space="preserve">  New Users — Dec-27</t>
         </is>
       </c>
       <c r="B112" s="8" t="n">
-        <v>18000</v>
+        <v>20000</v>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
@@ -2334,11 +2334,11 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Feb-28</t>
+          <t xml:space="preserve">  New Users — Jan-28</t>
         </is>
       </c>
       <c r="B113" s="8" t="n">
-        <v>16000</v>
+        <v>18000</v>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
@@ -2354,87 +2354,85 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  New Users — Feb-28</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="n">
+        <v>16000</v>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  New Users — Mar-28</t>
         </is>
       </c>
-      <c r="B114" s="8" t="n">
+      <c r="B115" s="8" t="n">
         <v>13000</v>
       </c>
-      <c r="C114" s="5" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>users</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>Monthly new user target</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="inlineStr"/>
-    </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
+      <c r="A116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>CASH</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="3" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
         <is>
           <t>Starting Cash</t>
         </is>
       </c>
-      <c r="B117" s="8" t="n">
+      <c r="B118" s="8" t="n">
         <v>1000</v>
       </c>
-      <c r="C117" s="5" t="inlineStr">
+      <c r="C118" s="5" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
+      <c r="D118" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
         <is>
           <t>MARKET REFERENCE (informational)</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="3" t="inlineStr">
-        <is>
-          <t>TAM — Fantasy Sports (2025)</t>
-        </is>
-      </c>
-      <c r="B120" s="5" t="inlineStr">
-        <is>
-          <t>$32B+</t>
-        </is>
-      </c>
-      <c r="C120" s="5" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>Mordor Intelligence</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>SAM — Fantasy Hockey Global</t>
+          <t>TAM — Fantasy Sports (2025)</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>$1-2B</t>
+          <t>$32B+</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
@@ -2444,95 +2442,95 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Industry estimates</t>
+          <t>Mordor Intelligence</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Active Fantasy Hockey Players (NA)</t>
+          <t>SAM — Fantasy Hockey Global</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>5,800,000</t>
+          <t>$1-2B</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>Users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>FSGA industry data</t>
+          <t>Industry estimates</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
+          <t>Active Fantasy Hockey Players (NA)</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>5,800,000</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>FSGA industry data</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
           <t>NHL Fantasy CAGR</t>
         </is>
       </c>
-      <c r="B123" s="5" t="inlineStr">
+      <c r="B124" s="5" t="inlineStr">
         <is>
           <t>14.6%</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C124" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr">
+      <c r="D124" t="inlineStr">
         <is>
           <t>Mordor Intelligence</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="inlineStr"/>
-    </row>
     <row r="125">
-      <c r="A125" s="2" t="inlineStr">
+      <c r="A125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
         <is>
           <t>BENCHMARKS</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="3" t="inlineStr">
-        <is>
-          <t>Mobile Freemium Median</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="inlineStr">
-        <is>
-          <t>2.18%</t>
-        </is>
-      </c>
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>RevenueCat 2025</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Sleeper Annual Retention</t>
+          <t>Mobile Freemium Median</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>2.18%</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
@@ -2542,56 +2540,78 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Sleeper Series C PR</t>
+          <t>RevenueCat 2025</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>DraftKings/FanDuel CAC</t>
+          <t>Sleeper Annual Retention</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>$200-350</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>BusinessOfApps</t>
+          <t>Sleeper Series C PR</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
+          <t>DraftKings/FanDuel CAC</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>$200-350</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>BusinessOfApps</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
           <t>NA Mobile CPI</t>
         </is>
       </c>
-      <c r="B129" s="5" t="inlineStr">
+      <c r="B130" s="5" t="inlineStr">
         <is>
           <t>$5.28</t>
         </is>
       </c>
-      <c r="C129" s="5" t="inlineStr">
+      <c r="C130" s="5" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="D130" t="inlineStr">
         <is>
           <t>BusinessOfApps</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="11" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
         <is>
           <t>Edit any yellow cell above to recalculate the entire model.</t>
         </is>
@@ -2899,99 +2919,99 @@
         </is>
       </c>
       <c r="B3" s="15">
-        <f>Assumptions!$B$91</f>
+        <f>Assumptions!$B$92</f>
         <v/>
       </c>
       <c r="C3" s="15">
-        <f>Assumptions!$B$92</f>
+        <f>Assumptions!$B$93</f>
         <v/>
       </c>
       <c r="D3" s="15">
-        <f>Assumptions!$B$93</f>
+        <f>Assumptions!$B$94</f>
         <v/>
       </c>
       <c r="E3" s="15">
-        <f>Assumptions!$B$94</f>
+        <f>Assumptions!$B$95</f>
         <v/>
       </c>
       <c r="F3" s="15">
-        <f>Assumptions!$B$95</f>
+        <f>Assumptions!$B$96</f>
         <v/>
       </c>
       <c r="G3" s="15">
-        <f>Assumptions!$B$96</f>
+        <f>Assumptions!$B$97</f>
         <v/>
       </c>
       <c r="H3" s="15">
-        <f>Assumptions!$B$97</f>
+        <f>Assumptions!$B$98</f>
         <v/>
       </c>
       <c r="I3" s="15">
-        <f>Assumptions!$B$98</f>
+        <f>Assumptions!$B$99</f>
         <v/>
       </c>
       <c r="J3" s="15">
-        <f>Assumptions!$B$99</f>
+        <f>Assumptions!$B$100</f>
         <v/>
       </c>
       <c r="K3" s="15">
-        <f>Assumptions!$B$100</f>
+        <f>Assumptions!$B$101</f>
         <v/>
       </c>
       <c r="L3" s="15">
-        <f>Assumptions!$B$101</f>
+        <f>Assumptions!$B$102</f>
         <v/>
       </c>
       <c r="M3" s="15">
-        <f>Assumptions!$B$102</f>
+        <f>Assumptions!$B$103</f>
         <v/>
       </c>
       <c r="N3" s="15">
-        <f>Assumptions!$B$103</f>
+        <f>Assumptions!$B$104</f>
         <v/>
       </c>
       <c r="O3" s="15">
-        <f>Assumptions!$B$104</f>
+        <f>Assumptions!$B$105</f>
         <v/>
       </c>
       <c r="P3" s="15">
-        <f>Assumptions!$B$105</f>
+        <f>Assumptions!$B$106</f>
         <v/>
       </c>
       <c r="Q3" s="15">
-        <f>Assumptions!$B$106</f>
+        <f>Assumptions!$B$107</f>
         <v/>
       </c>
       <c r="R3" s="15">
-        <f>Assumptions!$B$107</f>
+        <f>Assumptions!$B$108</f>
         <v/>
       </c>
       <c r="S3" s="15">
-        <f>Assumptions!$B$108</f>
+        <f>Assumptions!$B$109</f>
         <v/>
       </c>
       <c r="T3" s="15">
-        <f>Assumptions!$B$109</f>
+        <f>Assumptions!$B$110</f>
         <v/>
       </c>
       <c r="U3" s="15">
-        <f>Assumptions!$B$110</f>
+        <f>Assumptions!$B$111</f>
         <v/>
       </c>
       <c r="V3" s="15">
-        <f>Assumptions!$B$111</f>
+        <f>Assumptions!$B$112</f>
         <v/>
       </c>
       <c r="W3" s="15">
-        <f>Assumptions!$B$112</f>
+        <f>Assumptions!$B$113</f>
         <v/>
       </c>
       <c r="X3" s="15">
-        <f>Assumptions!$B$113</f>
+        <f>Assumptions!$B$114</f>
         <v/>
       </c>
       <c r="Y3" s="15">
-        <f>Assumptions!$B$114</f>
+        <f>Assumptions!$B$115</f>
         <v/>
       </c>
     </row>
@@ -9593,99 +9613,99 @@
         </is>
       </c>
       <c r="B22" s="15">
-        <f>IF('User Growth'!B20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!B20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="C22" s="15">
-        <f>IF('User Growth'!C20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!C20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="D22" s="15">
-        <f>IF('User Growth'!D20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!D20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="E22" s="15">
-        <f>IF('User Growth'!E20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!E20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="F22" s="15">
-        <f>IF('User Growth'!F20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!F20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="G22" s="15">
-        <f>IF('User Growth'!G20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!G20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="H22" s="15">
-        <f>IF('User Growth'!H20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!H20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="I22" s="15">
-        <f>IF('User Growth'!I20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!I20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="J22" s="15">
-        <f>IF('User Growth'!J20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!J20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="K22" s="15">
-        <f>IF('User Growth'!K20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!K20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="L22" s="15">
-        <f>IF('User Growth'!L20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!L20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="M22" s="15">
-        <f>IF('User Growth'!M20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!M20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="N22" s="15">
-        <f>IF('User Growth'!N20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!N20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="O22" s="15">
-        <f>IF('User Growth'!O20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!O20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="P22" s="15">
-        <f>IF('User Growth'!P20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!P20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="Q22" s="15">
-        <f>IF('User Growth'!Q20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!Q20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="R22" s="15">
-        <f>IF('User Growth'!R20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!R20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="S22" s="15">
-        <f>IF('User Growth'!S20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!S20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="T22" s="15">
-        <f>IF('User Growth'!T20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!T20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="U22" s="15">
-        <f>IF('User Growth'!U20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!U20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="V22" s="15">
-        <f>IF('User Growth'!V20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!V20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="W22" s="15">
-        <f>IF('User Growth'!W20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!W20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="X22" s="15">
-        <f>IF('User Growth'!X20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!X20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
       <c r="Y22" s="15">
-        <f>IF('User Growth'!Y20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88,0)</f>
+        <f>IF('User Growth'!Y20&gt;=Assumptions!$B$85,Assumptions!$B$86+Assumptions!$B$87+Assumptions!$B$88+Assumptions!$B$89,0)</f>
         <v/>
       </c>
     </row>
@@ -11996,7 +12016,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Assumptions!$B$117</f>
+        <f>Assumptions!$B$118</f>
         <v/>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -12133,7 +12153,7 @@
         </is>
       </c>
       <c r="B4" s="18">
-        <f>Assumptions!$B$117+B3</f>
+        <f>Assumptions!$B$118+B3</f>
         <v/>
       </c>
       <c r="C4" s="18">
@@ -13305,7 +13325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -13694,7 +13714,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>DFS REGULATORY</t>
+          <t>DFS REGULATORY — CANADA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -13702,316 +13722,338 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>State-by-state DFS licensing</t>
+          <t>Canadian Criminal Code s.206 skill exemption</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Legal Sports Report — State DFS Laws</t>
+          <t>Criminal Code of Canada — Contest provisions</t>
         </is>
       </c>
       <c r="C32" s="28" t="inlineStr">
         <is>
-          <t>https://www.legalsportsreport.com/dfs-bill-tracker/</t>
+          <t>https://laws-lois.justice.gc.ca/eng/acts/c-46/page-46.html</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DFS compliance requirements</t>
+          <t>Ontario iGaming framework (2022+)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NYDFS DFS Regulations (example)</t>
+          <t>iGaming Ontario — Operator Registration</t>
         </is>
       </c>
       <c r="C33" s="28" t="inlineStr">
         <is>
-          <t>https://www.dfs.ny.gov/industry_guidance/fantasy_sports</t>
+          <t>https://igamingontario.ca/en/operators</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Surety bond / insurance requirements</t>
+          <t>AGCO gaming registration requirements</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>State gaming commission requirements</t>
+          <t>Alcohol &amp; Gaming Commission of Ontario</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>https://www.agco.ca/igaming</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Typical state license cost $5K-$50K+</t>
+          <t>FINTRAC AML obligations for gaming</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Varies by state — NY, MA, VA most expensive</t>
+          <t>FINTRAC — Reporting Entity Requirements</t>
+        </is>
+      </c>
+      <c r="C35" s="28" t="inlineStr">
+        <is>
+          <t>https://fintrac-canafe.canada.ca/re-ed/intro-eng</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Provincial gaming oversight (AB/BC/QC)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Varies by province — nominal registration fees</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>MARKETING / CAC</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>DraftKings/FanDuel CAC $200-350</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>BusinessOfApps UA Costs</t>
-        </is>
-      </c>
-      <c r="C38" s="28" t="inlineStr">
-        <is>
-          <t>https://www.businessofapps.com/marketplace/user-acquisition/research/user-acquisition-costs/</t>
-        </is>
-      </c>
+      <c r="B38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>DraftKings/FanDuel CAC $200-350</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>BusinessOfApps UA Costs</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>https://www.businessofapps.com/marketplace/user-acquisition/research/user-acquisition-costs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>NA Mobile CPI $5.28</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>BusinessOfApps UA Costs</t>
         </is>
       </c>
-      <c r="C39" s="28" t="inlineStr">
+      <c r="C40" s="28" t="inlineStr">
         <is>
           <t>https://www.businessofapps.com/marketplace/user-acquisition/research/user-acquisition-costs/</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr"/>
-    </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>MARKET DATA</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Fantasy sports market $32B, 14.1% CAGR</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Mordor Intelligence</t>
-        </is>
-      </c>
-      <c r="C42" s="28" t="inlineStr">
-        <is>
-          <t>https://www.mordorintelligence.com/industry-reports/north-america-fantasy-sports-market</t>
-        </is>
-      </c>
+      <c r="B42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Fantasy sports market $32B, 14.1% CAGR</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Mordor Intelligence</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="inlineStr">
+        <is>
+          <t>https://www.mordorintelligence.com/industry-reports/north-america-fantasy-sports-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>Sleeper $40M Series C, 3M+ users</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>PR Newswire</t>
         </is>
       </c>
-      <c r="C43" s="28" t="inlineStr">
+      <c r="C44" s="28" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/fantasy-sports-app-sleeper-raises-40-million-doubles-user-base-in-2021-301379179.html</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>METHODOLOGY NOTES</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>User growth model</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Bottom-up monthly cohort model with seasonal multipliers</t>
-        </is>
-      </c>
+      <c r="B46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Conversion timing</t>
+          <t>User growth model</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>In-season 1.8x multiplier, off-season 0.4x</t>
+          <t>Bottom-up monthly cohort model with seasonal multipliers</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Churn model</t>
+          <t>Conversion timing</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Monthly churn with seasonal variation (in vs off-season)</t>
+          <t>In-season 1.8x multiplier, off-season 0.4x</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Revenue recognition</t>
+          <t>Churn model</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Subscription recognized monthly; annual billing amortized</t>
+          <t>Monthly churn with seasonal variation (in vs off-season)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Marketing timing</t>
+          <t>Revenue recognition</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>No marketing spend pre-launch; starts at configurable launch month</t>
+          <t>Subscription recognized monthly; annual billing amortized</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Platform fee allocation</t>
+          <t>Marketing timing</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>70% mobile (60/40 iOS/Android), 30% web (Stripe)</t>
+          <t>No marketing spend pre-launch; starts at configurable launch month</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>COGS scaling</t>
+          <t>Platform fee allocation</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Supabase upgrades at 50K users; Claude API scales per-query</t>
+          <t>70% mobile (60/40 iOS/Android), 30% web (Stripe)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DFS regulatory</t>
+          <t>COGS scaling</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>State licensing + compliance + insurance triggers at 100K users</t>
+          <t>Supabase upgrades at 50K users; Claude API scales per-query</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>DFS regulatory (Canada)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ontario iGaming + provincial fees + FINTRAC AML triggers at 100K users</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>DFS launch</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Month 19 (Oct 2027) per product roadmap</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-    </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>DYNAMIC MODEL NOTE</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>All computed cells use Excel formulas</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Change any yellow input cell to recalculate instantly</t>
-        </is>
-      </c>
+      <c r="B57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Input cells on Assumptions tab</t>
+          <t>All computed cells use Excel formulas</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>All model inputs: pricing, rates, costs, AND monthly new user targets</t>
+          <t>Change any yellow input cell to recalculate instantly</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>Input cells on Assumptions tab</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>All model inputs: pricing, rates, costs, AND monthly new user targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Input cells on COGS tab</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Monthly conference/travel costs</t>
         </is>

</xml_diff>

<commit_message>
Add US DFS expansion toggle with state-by-state licensing costs
19 states modeled with actual Year 1 and annual renewal fees (NY $500K Y1
down to $5K states). Includes compliance overhead (legal counsel, geolocation,
audits, responsible gaming, NY revenue tax). Toggle defaults to 99 (OFF) —
set to a month index (0-23) on Assumptions tab to activate.

Year 1 all-in: ~$1.13M | Year 2+: ~$595K/yr

https://claude.ai/code/session_01DWcMBbfjeLfgrVr7i298sA
</commit_message>
<xml_diff>
--- a/docs/Citrus_Business_Model.xlsx
+++ b/docs/Citrus_Business_Model.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2447,533 +2447,568 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>USER GROWTH / ACQUISITION (Monthly New Users)</t>
+          <t>US DFS EXPANSION (Toggle)</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Apr-26</t>
+          <t>US Expansion Launch Month</t>
         </is>
       </c>
       <c r="B121" s="7" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>0-based</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>Set to 99 = OFF; e.g. 18 = Oct-27</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  New Users — May-26</t>
-        </is>
-      </c>
-      <c r="B122" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>users</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>Monthly new user target</t>
-        </is>
-      </c>
+      <c r="A122" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  New Users — Jun-26</t>
-        </is>
-      </c>
-      <c r="B123" s="7" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>users</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>Monthly new user target</t>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STATE-BY-STATE LICENSING FEES (Year 1 / Annual)</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jul-26</t>
+          <t xml:space="preserve">  New York — Year 1</t>
         </is>
       </c>
       <c r="B124" s="7" t="n">
-        <v>3000</v>
+        <v>500000</v>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>NY Gaming Commission — most expensive state</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Aug-26</t>
+          <t xml:space="preserve">  New York — Annual Renewal</t>
         </is>
       </c>
       <c r="B125" s="7" t="n">
-        <v>6000</v>
+        <v>50000</v>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>NY Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Sep-26</t>
+          <t xml:space="preserve">  Massachusetts — Year 1</t>
         </is>
       </c>
       <c r="B126" s="7" t="n">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>MA Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Oct-26</t>
+          <t xml:space="preserve">  Massachusetts — Annual Renewal</t>
         </is>
       </c>
       <c r="B127" s="7" t="n">
-        <v>8000</v>
+        <v>50000</v>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>MA Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Nov-26</t>
+          <t xml:space="preserve">  Virginia — Year 1</t>
         </is>
       </c>
       <c r="B128" s="7" t="n">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>VA Lottery</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Dec-26</t>
+          <t xml:space="preserve">  Virginia — Annual Renewal</t>
         </is>
       </c>
       <c r="B129" s="7" t="n">
-        <v>3000</v>
+        <v>50000</v>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>VA Lottery</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jan-27</t>
+          <t xml:space="preserve">  Tennessee — Year 1</t>
         </is>
       </c>
       <c r="B130" s="7" t="n">
-        <v>2500</v>
+        <v>50000</v>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>TN Secretary of State</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Feb-27</t>
+          <t xml:space="preserve">  Tennessee — Annual Renewal</t>
         </is>
       </c>
       <c r="B131" s="7" t="n">
-        <v>2000</v>
+        <v>50000</v>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>TN Secretary of State</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Mar-27</t>
+          <t xml:space="preserve">  Indiana — Year 1</t>
         </is>
       </c>
       <c r="B132" s="7" t="n">
-        <v>1500</v>
+        <v>50000</v>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>IN Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Apr-27</t>
+          <t xml:space="preserve">  Indiana — Annual Renewal</t>
         </is>
       </c>
       <c r="B133" s="7" t="n">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>IN Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — May-27</t>
+          <t xml:space="preserve">  Pennsylvania — Year 1</t>
         </is>
       </c>
       <c r="B134" s="7" t="n">
-        <v>2000</v>
+        <v>50000</v>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>PA Gaming Control Board</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jun-27</t>
+          <t xml:space="preserve">  Pennsylvania — Annual Renewal</t>
         </is>
       </c>
       <c r="B135" s="7" t="n">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>PA Gaming Control Board</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jul-27</t>
+          <t xml:space="preserve">  Connecticut — Year 1</t>
         </is>
       </c>
       <c r="B136" s="7" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>CT Dept Consumer Protection</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Aug-27</t>
+          <t xml:space="preserve">  Connecticut — Annual Renewal</t>
         </is>
       </c>
       <c r="B137" s="7" t="n">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>CT Dept Consumer Protection</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Sep-27</t>
+          <t xml:space="preserve">  Colorado — Year 1</t>
         </is>
       </c>
       <c r="B138" s="7" t="n">
-        <v>12000</v>
+        <v>10000</v>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>CO Dept of Revenue</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Oct-27</t>
+          <t xml:space="preserve">  Colorado — Annual Renewal</t>
         </is>
       </c>
       <c r="B139" s="7" t="n">
-        <v>17000</v>
+        <v>10000</v>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>CO Dept of Revenue</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Nov-27</t>
+          <t xml:space="preserve">  Illinois — Year 1</t>
         </is>
       </c>
       <c r="B140" s="7" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>IL Gaming Board</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Dec-27</t>
+          <t xml:space="preserve">  Illinois — Annual Renewal</t>
         </is>
       </c>
       <c r="B141" s="7" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>IL Gaming Board</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Jan-28</t>
+          <t xml:space="preserve">  Missouri — Year 1</t>
         </is>
       </c>
       <c r="B142" s="7" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>MO Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Feb-28</t>
+          <t xml:space="preserve">  Missouri — Annual Renewal</t>
         </is>
       </c>
       <c r="B143" s="7" t="n">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>MO Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Users — Mar-28</t>
+          <t xml:space="preserve">  Oregon — Year 1</t>
         </is>
       </c>
       <c r="B144" s="7" t="n">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Monthly new user target</t>
+          <t>OR Dept of Justice</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr"/>
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Oregon — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>OR Dept of Justice</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="inlineStr">
-        <is>
-          <t>CASH</t>
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Maryland — Year 1</t>
+        </is>
+      </c>
+      <c r="B146" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>MD Lottery &amp; Gaming</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Starting Cash</t>
+          <t xml:space="preserve">  Maryland — Annual Renewal</t>
         </is>
       </c>
       <c r="B147" s="7" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>MD Lottery &amp; Gaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kansas — Year 1</t>
+        </is>
+      </c>
+      <c r="B148" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>KS Attorney General</t>
+        </is>
+      </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>MARKET REFERENCE (informational)</t>
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kansas — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B149" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>KS Attorney General</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>TAM — Fantasy Sports (2025)</t>
-        </is>
-      </c>
-      <c r="B150" s="5" t="inlineStr">
-        <is>
-          <t>$32B+</t>
-        </is>
+          <t xml:space="preserve">  Vermont — Year 1</t>
+        </is>
+      </c>
+      <c r="B150" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
@@ -2982,140 +3017,158 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Mordor Intelligence</t>
+          <t>VT Attorney General</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>SAM — Fantasy Hockey Global</t>
-        </is>
-      </c>
-      <c r="B151" s="5" t="inlineStr">
-        <is>
-          <t>$1-2B</t>
-        </is>
+          <t xml:space="preserve">  Vermont — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B151" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Industry estimates</t>
+          <t>VT Attorney General</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Active Fantasy Hockey Players (NA)</t>
-        </is>
-      </c>
-      <c r="B152" s="5" t="inlineStr">
-        <is>
-          <t>5,800,000</t>
-        </is>
+          <t xml:space="preserve">  Arkansas — Year 1</t>
+        </is>
+      </c>
+      <c r="B152" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C152" s="5" t="inlineStr">
         <is>
-          <t>Users</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>FSGA industry data</t>
+          <t>AR Dept Finance &amp; Admin</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>NHL Fantasy CAGR</t>
-        </is>
-      </c>
-      <c r="B153" s="5" t="inlineStr">
-        <is>
-          <t>14.6%</t>
-        </is>
+          <t xml:space="preserve">  Arkansas — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B153" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Mordor Intelligence</t>
+          <t>AR Dept Finance &amp; Admin</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr"/>
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mississippi — Year 1</t>
+        </is>
+      </c>
+      <c r="B154" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>MS Gaming Commission</t>
+        </is>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>BENCHMARKS</t>
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mississippi — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B155" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>MS Gaming Commission</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>Mobile Freemium Median</t>
-        </is>
-      </c>
-      <c r="B156" s="5" t="inlineStr">
-        <is>
-          <t>2.18%</t>
-        </is>
+          <t xml:space="preserve">  New Hampshire — Year 1</t>
+        </is>
+      </c>
+      <c r="B156" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>RevenueCat 2025</t>
+          <t>NH Lottery Commission</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Sleeper Annual Retention</t>
-        </is>
-      </c>
-      <c r="B157" s="5" t="inlineStr">
-        <is>
-          <t>75%</t>
-        </is>
+          <t xml:space="preserve">  New Hampshire — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B157" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD/yr</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Sleeper Series C PR</t>
+          <t>NH Lottery Commission</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>DraftKings/FanDuel CAC</t>
-        </is>
-      </c>
-      <c r="B158" s="5" t="inlineStr">
-        <is>
-          <t>$200-350</t>
-        </is>
+          <t xml:space="preserve">  Delaware — Year 1</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="n">
+        <v>5000</v>
       </c>
       <c r="C158" s="5" t="inlineStr">
         <is>
@@ -3124,34 +3177,951 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>BusinessOfApps</t>
+          <t>DE Dept of Finance</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Delaware — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B159" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>DE Dept of Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rhode Island — Year 1</t>
+        </is>
+      </c>
+      <c r="B160" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>RI DBR</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rhode Island — Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>RI DBR</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  US COMPLIANCE OVERHEAD (Annual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Multi-State Legal Counsel</t>
+        </is>
+      </c>
+      <c r="B164" s="7" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>DFS compliance firm</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Geolocation Vendor (GeoComply etc.)</t>
+        </is>
+      </c>
+      <c r="B165" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Block banned states, verify regulated</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Independent Financial Audit</t>
+        </is>
+      </c>
+      <c r="B166" s="7" t="n">
+        <v>35000</v>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Required by most regulated states</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Responsible Gaming Program</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Self-exclusion, limits, reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  State Reporting &amp; Filings</t>
+        </is>
+      </c>
+      <c r="B168" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Annual filings, revenue reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Background Checks (Key Personnel)</t>
+        </is>
+      </c>
+      <c r="B169" s="7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Required for all licensed states</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NY Revenue Tax Rate</t>
+        </is>
+      </c>
+      <c r="B170" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>~15% of DFS revenue from NY users</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Est. NY Revenue Share (% of total)</t>
+        </is>
+      </c>
+      <c r="B171" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>NY ~12% of US DFS market</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>USER GROWTH / ACQUISITION (Monthly New Users)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Apr-26</t>
+        </is>
+      </c>
+      <c r="B174" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — May-26</t>
+        </is>
+      </c>
+      <c r="B175" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Jun-26</t>
+        </is>
+      </c>
+      <c r="B176" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Jul-26</t>
+        </is>
+      </c>
+      <c r="B177" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Aug-26</t>
+        </is>
+      </c>
+      <c r="B178" s="7" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Sep-26</t>
+        </is>
+      </c>
+      <c r="B179" s="7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Oct-26</t>
+        </is>
+      </c>
+      <c r="B180" s="7" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Nov-26</t>
+        </is>
+      </c>
+      <c r="B181" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Dec-26</t>
+        </is>
+      </c>
+      <c r="B182" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Jan-27</t>
+        </is>
+      </c>
+      <c r="B183" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Feb-27</t>
+        </is>
+      </c>
+      <c r="B184" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Mar-27</t>
+        </is>
+      </c>
+      <c r="B185" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Apr-27</t>
+        </is>
+      </c>
+      <c r="B186" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — May-27</t>
+        </is>
+      </c>
+      <c r="B187" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Jun-27</t>
+        </is>
+      </c>
+      <c r="B188" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Jul-27</t>
+        </is>
+      </c>
+      <c r="B189" s="7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Aug-27</t>
+        </is>
+      </c>
+      <c r="B190" s="7" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Sep-27</t>
+        </is>
+      </c>
+      <c r="B191" s="7" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Oct-27</t>
+        </is>
+      </c>
+      <c r="B192" s="7" t="n">
+        <v>17000</v>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Nov-27</t>
+        </is>
+      </c>
+      <c r="B193" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Dec-27</t>
+        </is>
+      </c>
+      <c r="B194" s="7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Jan-28</t>
+        </is>
+      </c>
+      <c r="B195" s="7" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Feb-28</t>
+        </is>
+      </c>
+      <c r="B196" s="7" t="n">
+        <v>16000</v>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  New Users — Mar-28</t>
+        </is>
+      </c>
+      <c r="B197" s="7" t="n">
+        <v>13000</v>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Monthly new user target</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>Starting Cash</t>
+        </is>
+      </c>
+      <c r="B200" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>MARKET REFERENCE (informational)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>TAM — Fantasy Sports (2025)</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>$32B+</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Mordor Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>SAM — Fantasy Hockey Global</t>
+        </is>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>$1-2B</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Industry estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>Active Fantasy Hockey Players (NA)</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>5,800,000</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>FSGA industry data</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>NHL Fantasy CAGR</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Mordor Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>BENCHMARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>Mobile Freemium Median</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>2.18%</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>RevenueCat 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>Sleeper Annual Retention</t>
+        </is>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Sleeper Series C PR</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>DraftKings/FanDuel CAC</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="inlineStr">
+        <is>
+          <t>$200-350</t>
+        </is>
+      </c>
+      <c r="C211" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>BusinessOfApps</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
           <t>NA Mobile CPI</t>
         </is>
       </c>
-      <c r="B159" s="5" t="inlineStr">
+      <c r="B212" s="5" t="inlineStr">
         <is>
           <t>$5.28</t>
         </is>
       </c>
-      <c r="C159" s="5" t="inlineStr">
+      <c r="C212" s="5" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr">
+      <c r="D212" t="inlineStr">
         <is>
           <t>BusinessOfApps</t>
         </is>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" s="11" t="inlineStr">
+    <row r="214">
+      <c r="A214" s="11" t="inlineStr">
         <is>
           <t>Edit any yellow cell above to recalculate the entire model.</t>
         </is>
@@ -3459,99 +4429,99 @@
         </is>
       </c>
       <c r="B3" s="15">
-        <f>Assumptions!$B$121</f>
+        <f>Assumptions!$B$174</f>
         <v/>
       </c>
       <c r="C3" s="15">
-        <f>Assumptions!$B$122</f>
+        <f>Assumptions!$B$175</f>
         <v/>
       </c>
       <c r="D3" s="15">
-        <f>Assumptions!$B$123</f>
+        <f>Assumptions!$B$176</f>
         <v/>
       </c>
       <c r="E3" s="15">
-        <f>Assumptions!$B$124</f>
+        <f>Assumptions!$B$177</f>
         <v/>
       </c>
       <c r="F3" s="15">
-        <f>Assumptions!$B$125</f>
+        <f>Assumptions!$B$178</f>
         <v/>
       </c>
       <c r="G3" s="15">
-        <f>Assumptions!$B$126</f>
+        <f>Assumptions!$B$179</f>
         <v/>
       </c>
       <c r="H3" s="15">
-        <f>Assumptions!$B$127</f>
+        <f>Assumptions!$B$180</f>
         <v/>
       </c>
       <c r="I3" s="15">
-        <f>Assumptions!$B$128</f>
+        <f>Assumptions!$B$181</f>
         <v/>
       </c>
       <c r="J3" s="15">
-        <f>Assumptions!$B$129</f>
+        <f>Assumptions!$B$182</f>
         <v/>
       </c>
       <c r="K3" s="15">
-        <f>Assumptions!$B$130</f>
+        <f>Assumptions!$B$183</f>
         <v/>
       </c>
       <c r="L3" s="15">
-        <f>Assumptions!$B$131</f>
+        <f>Assumptions!$B$184</f>
         <v/>
       </c>
       <c r="M3" s="15">
-        <f>Assumptions!$B$132</f>
+        <f>Assumptions!$B$185</f>
         <v/>
       </c>
       <c r="N3" s="15">
-        <f>Assumptions!$B$133</f>
+        <f>Assumptions!$B$186</f>
         <v/>
       </c>
       <c r="O3" s="15">
-        <f>Assumptions!$B$134</f>
+        <f>Assumptions!$B$187</f>
         <v/>
       </c>
       <c r="P3" s="15">
-        <f>Assumptions!$B$135</f>
+        <f>Assumptions!$B$188</f>
         <v/>
       </c>
       <c r="Q3" s="15">
-        <f>Assumptions!$B$136</f>
+        <f>Assumptions!$B$189</f>
         <v/>
       </c>
       <c r="R3" s="15">
-        <f>Assumptions!$B$137</f>
+        <f>Assumptions!$B$190</f>
         <v/>
       </c>
       <c r="S3" s="15">
-        <f>Assumptions!$B$138</f>
+        <f>Assumptions!$B$191</f>
         <v/>
       </c>
       <c r="T3" s="15">
-        <f>Assumptions!$B$139</f>
+        <f>Assumptions!$B$192</f>
         <v/>
       </c>
       <c r="U3" s="15">
-        <f>Assumptions!$B$140</f>
+        <f>Assumptions!$B$193</f>
         <v/>
       </c>
       <c r="V3" s="15">
-        <f>Assumptions!$B$141</f>
+        <f>Assumptions!$B$194</f>
         <v/>
       </c>
       <c r="W3" s="15">
-        <f>Assumptions!$B$142</f>
+        <f>Assumptions!$B$195</f>
         <v/>
       </c>
       <c r="X3" s="15">
-        <f>Assumptions!$B$143</f>
+        <f>Assumptions!$B$196</f>
         <v/>
       </c>
       <c r="Y3" s="15">
-        <f>Assumptions!$B$144</f>
+        <f>Assumptions!$B$197</f>
         <v/>
       </c>
     </row>
@@ -8622,7 +9592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y36"/>
+  <dimension ref="A1:Y39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -10149,7 +11119,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    DFS Regulatory / Licensing</t>
+          <t xml:space="preserve">    DFS Regulatory — Canada</t>
         </is>
       </c>
       <c r="B22" s="15">
@@ -10252,910 +11222,1219 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Apple Developer Program</t>
-        </is>
-      </c>
-      <c r="B23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="C23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="D23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="E23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="F23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="G23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="H23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="I23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="J23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="K23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="L23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="M23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="N23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="O23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="P23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="Q23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="R23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="S23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="T23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="U23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="V23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="W23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="X23" s="19">
-        <f>Assumptions!$B$70/12</f>
-        <v/>
-      </c>
-      <c r="Y23" s="19">
-        <f>Assumptions!$B$70/12</f>
+          <t xml:space="preserve">    US DFS Licensing (State-by-State)</t>
+        </is>
+      </c>
+      <c r="B23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="C23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="D23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="H23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="I23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="J23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="K23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="L23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="M23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="N23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="O23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="P23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="R23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="S23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="T23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="U23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="V23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="W23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="X23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
+        <v/>
+      </c>
+      <c r="Y23" s="15">
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,IF(COLUMN()-2-Assumptions!$B$121&lt;12,Assumptions!$B$124/12+Assumptions!$B$126/12+Assumptions!$B$128/12+Assumptions!$B$130/12+Assumptions!$B$132/12+Assumptions!$B$134/12+Assumptions!$B$136/12+Assumptions!$B$138/12+Assumptions!$B$140/12+Assumptions!$B$142/12+Assumptions!$B$144/12+Assumptions!$B$146/12+Assumptions!$B$148/12+Assumptions!$B$150/12+Assumptions!$B$152/12+Assumptions!$B$154/12+Assumptions!$B$156/12+Assumptions!$B$158/12+Assumptions!$B$160/12,Assumptions!$B$125/12+Assumptions!$B$127/12+Assumptions!$B$129/12+Assumptions!$B$131/12+Assumptions!$B$133/12+Assumptions!$B$135/12+Assumptions!$B$137/12+Assumptions!$B$139/12+Assumptions!$B$141/12+Assumptions!$B$143/12+Assumptions!$B$145/12+Assumptions!$B$147/12+Assumptions!$B$149/12+Assumptions!$B$151/12+Assumptions!$B$153/12+Assumptions!$B$155/12+Assumptions!$B$157/12+Assumptions!$B$159/12+Assumptions!$B$161/12),0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Google Play Registration</t>
+          <t xml:space="preserve">    US DFS Compliance Overhead</t>
         </is>
       </c>
       <c r="B24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!B20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="C24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!C20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="D24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!D20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="E24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!E20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="F24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!F20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="G24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!G20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="H24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!H20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="I24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!I20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="J24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!J20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="K24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!K20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="L24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!L20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="M24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!M20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="N24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!N20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="O24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!O20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="P24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!P20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="Q24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!Q20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="R24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!R20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="S24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!S20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="T24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!T20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="U24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!U20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="V24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!V20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="W24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!W20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="X24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!X20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
       <c r="Y24" s="15">
-        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <f>IF(COLUMN()-2&gt;=Assumptions!$B$121,Assumptions!$B$164/12+Assumptions!$B$165/12+Assumptions!$B$166/12+Assumptions!$B$167/12+Assumptions!$B$168/12+Assumptions!$B$169/12+Revenue!Y20*Assumptions!$B$171*Assumptions!$B$170,0)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
+          <t xml:space="preserve">    Total US DFS Expansion</t>
+        </is>
+      </c>
+      <c r="B25" s="18">
+        <f>B23+B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="18">
+        <f>C23+C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="18">
+        <f>D23+D24</f>
+        <v/>
+      </c>
+      <c r="E25" s="18">
+        <f>E23+E24</f>
+        <v/>
+      </c>
+      <c r="F25" s="18">
+        <f>F23+F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="18">
+        <f>G23+G24</f>
+        <v/>
+      </c>
+      <c r="H25" s="18">
+        <f>H23+H24</f>
+        <v/>
+      </c>
+      <c r="I25" s="18">
+        <f>I23+I24</f>
+        <v/>
+      </c>
+      <c r="J25" s="18">
+        <f>J23+J24</f>
+        <v/>
+      </c>
+      <c r="K25" s="18">
+        <f>K23+K24</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>L23+L24</f>
+        <v/>
+      </c>
+      <c r="M25" s="18">
+        <f>M23+M24</f>
+        <v/>
+      </c>
+      <c r="N25" s="18">
+        <f>N23+N24</f>
+        <v/>
+      </c>
+      <c r="O25" s="18">
+        <f>O23+O24</f>
+        <v/>
+      </c>
+      <c r="P25" s="18">
+        <f>P23+P24</f>
+        <v/>
+      </c>
+      <c r="Q25" s="18">
+        <f>Q23+Q24</f>
+        <v/>
+      </c>
+      <c r="R25" s="18">
+        <f>R23+R24</f>
+        <v/>
+      </c>
+      <c r="S25" s="18">
+        <f>S23+S24</f>
+        <v/>
+      </c>
+      <c r="T25" s="18">
+        <f>T23+T24</f>
+        <v/>
+      </c>
+      <c r="U25" s="18">
+        <f>U23+U24</f>
+        <v/>
+      </c>
+      <c r="V25" s="18">
+        <f>V23+V24</f>
+        <v/>
+      </c>
+      <c r="W25" s="18">
+        <f>W23+W24</f>
+        <v/>
+      </c>
+      <c r="X25" s="18">
+        <f>X23+X24</f>
+        <v/>
+      </c>
+      <c r="Y25" s="18">
+        <f>Y23+Y24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Apple Developer Program</t>
+        </is>
+      </c>
+      <c r="B26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="C26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="D26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="E26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="F26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="G26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="H26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="I26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="J26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="K26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="L26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="M26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="N26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="O26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="P26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="Q26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="R26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="S26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="T26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="U26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="V26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="W26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="X26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+      <c r="Y26" s="19">
+        <f>Assumptions!$B$70/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Google Play Registration</t>
+        </is>
+      </c>
+      <c r="B27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="E27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="F27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="H27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="I27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="J27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="K27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="M27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="N27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="O27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="P27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="R27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="S27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="T27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="U27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="V27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="W27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="X27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+      <c r="Y27" s="15">
+        <f>IF(COLUMN()=2,Assumptions!$B$71,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
           <t xml:space="preserve">    Total G&amp;A</t>
         </is>
       </c>
-      <c r="B25" s="18">
-        <f>B20+B21+B22+B23+B24</f>
-        <v/>
-      </c>
-      <c r="C25" s="18">
-        <f>C20+C21+C22+C23+C24</f>
-        <v/>
-      </c>
-      <c r="D25" s="18">
-        <f>D20+D21+D22+D23+D24</f>
-        <v/>
-      </c>
-      <c r="E25" s="18">
-        <f>E20+E21+E22+E23+E24</f>
-        <v/>
-      </c>
-      <c r="F25" s="18">
-        <f>F20+F21+F22+F23+F24</f>
-        <v/>
-      </c>
-      <c r="G25" s="18">
-        <f>G20+G21+G22+G23+G24</f>
-        <v/>
-      </c>
-      <c r="H25" s="18">
-        <f>H20+H21+H22+H23+H24</f>
-        <v/>
-      </c>
-      <c r="I25" s="18">
-        <f>I20+I21+I22+I23+I24</f>
-        <v/>
-      </c>
-      <c r="J25" s="18">
-        <f>J20+J21+J22+J23+J24</f>
-        <v/>
-      </c>
-      <c r="K25" s="18">
-        <f>K20+K21+K22+K23+K24</f>
-        <v/>
-      </c>
-      <c r="L25" s="18">
-        <f>L20+L21+L22+L23+L24</f>
-        <v/>
-      </c>
-      <c r="M25" s="18">
-        <f>M20+M21+M22+M23+M24</f>
-        <v/>
-      </c>
-      <c r="N25" s="18">
-        <f>N20+N21+N22+N23+N24</f>
-        <v/>
-      </c>
-      <c r="O25" s="18">
-        <f>O20+O21+O22+O23+O24</f>
-        <v/>
-      </c>
-      <c r="P25" s="18">
-        <f>P20+P21+P22+P23+P24</f>
-        <v/>
-      </c>
-      <c r="Q25" s="18">
-        <f>Q20+Q21+Q22+Q23+Q24</f>
-        <v/>
-      </c>
-      <c r="R25" s="18">
-        <f>R20+R21+R22+R23+R24</f>
-        <v/>
-      </c>
-      <c r="S25" s="18">
-        <f>S20+S21+S22+S23+S24</f>
-        <v/>
-      </c>
-      <c r="T25" s="18">
-        <f>T20+T21+T22+T23+T24</f>
-        <v/>
-      </c>
-      <c r="U25" s="18">
-        <f>U20+U21+U22+U23+U24</f>
-        <v/>
-      </c>
-      <c r="V25" s="18">
-        <f>V20+V21+V22+V23+V24</f>
-        <v/>
-      </c>
-      <c r="W25" s="18">
-        <f>W20+W21+W22+W23+W24</f>
-        <v/>
-      </c>
-      <c r="X25" s="18">
-        <f>X20+X21+X22+X23+X24</f>
-        <v/>
-      </c>
-      <c r="Y25" s="18">
-        <f>Y20+Y21+Y22+Y23+Y24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="B28" s="18">
+        <f>B20+B21+B22+B25+B26+B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="18">
+        <f>C20+C21+C22+C25+C26+C27</f>
+        <v/>
+      </c>
+      <c r="D28" s="18">
+        <f>D20+D21+D22+D25+D26+D27</f>
+        <v/>
+      </c>
+      <c r="E28" s="18">
+        <f>E20+E21+E22+E25+E26+E27</f>
+        <v/>
+      </c>
+      <c r="F28" s="18">
+        <f>F20+F21+F22+F25+F26+F27</f>
+        <v/>
+      </c>
+      <c r="G28" s="18">
+        <f>G20+G21+G22+G25+G26+G27</f>
+        <v/>
+      </c>
+      <c r="H28" s="18">
+        <f>H20+H21+H22+H25+H26+H27</f>
+        <v/>
+      </c>
+      <c r="I28" s="18">
+        <f>I20+I21+I22+I25+I26+I27</f>
+        <v/>
+      </c>
+      <c r="J28" s="18">
+        <f>J20+J21+J22+J25+J26+J27</f>
+        <v/>
+      </c>
+      <c r="K28" s="18">
+        <f>K20+K21+K22+K25+K26+K27</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
+        <f>L20+L21+L22+L25+L26+L27</f>
+        <v/>
+      </c>
+      <c r="M28" s="18">
+        <f>M20+M21+M22+M25+M26+M27</f>
+        <v/>
+      </c>
+      <c r="N28" s="18">
+        <f>N20+N21+N22+N25+N26+N27</f>
+        <v/>
+      </c>
+      <c r="O28" s="18">
+        <f>O20+O21+O22+O25+O26+O27</f>
+        <v/>
+      </c>
+      <c r="P28" s="18">
+        <f>P20+P21+P22+P25+P26+P27</f>
+        <v/>
+      </c>
+      <c r="Q28" s="18">
+        <f>Q20+Q21+Q22+Q25+Q26+Q27</f>
+        <v/>
+      </c>
+      <c r="R28" s="18">
+        <f>R20+R21+R22+R25+R26+R27</f>
+        <v/>
+      </c>
+      <c r="S28" s="18">
+        <f>S20+S21+S22+S25+S26+S27</f>
+        <v/>
+      </c>
+      <c r="T28" s="18">
+        <f>T20+T21+T22+T25+T26+T27</f>
+        <v/>
+      </c>
+      <c r="U28" s="18">
+        <f>U20+U21+U22+U25+U26+U27</f>
+        <v/>
+      </c>
+      <c r="V28" s="18">
+        <f>V20+V21+V22+V25+V26+V27</f>
+        <v/>
+      </c>
+      <c r="W28" s="18">
+        <f>W20+W21+W22+W25+W26+W27</f>
+        <v/>
+      </c>
+      <c r="X28" s="18">
+        <f>X20+X21+X22+X25+X26+X27</f>
+        <v/>
+      </c>
+      <c r="Y28" s="18">
+        <f>Y20+Y21+Y22+Y25+Y26+Y27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  CONFERENCE &amp; TRAVEL</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">    Conference Costs</t>
         </is>
       </c>
-      <c r="B28" s="20" t="n">
+      <c r="B31" s="20" t="n">
         <v>750</v>
       </c>
-      <c r="C28" s="20" t="n">
+      <c r="C31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D28" s="20" t="n">
+      <c r="D31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="20" t="n">
+      <c r="E31" s="20" t="n">
         <v>4500</v>
       </c>
-      <c r="F28" s="20" t="n">
+      <c r="F31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="20" t="n">
+      <c r="G31" s="20" t="n">
         <v>3500</v>
       </c>
-      <c r="H28" s="20" t="n">
+      <c r="H31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="20" t="n">
+      <c r="I31" s="20" t="n">
         <v>5000</v>
       </c>
-      <c r="J28" s="20" t="n">
+      <c r="J31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="20" t="n">
+      <c r="K31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="L28" s="20" t="n">
+      <c r="L31" s="20" t="n">
         <v>4000</v>
       </c>
-      <c r="M28" s="20" t="n">
+      <c r="M31" s="20" t="n">
         <v>5000</v>
       </c>
-      <c r="N28" s="20" t="n">
+      <c r="N31" s="20" t="n">
         <v>500</v>
       </c>
-      <c r="O28" s="20" t="n">
+      <c r="O31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="P28" s="20" t="n">
+      <c r="P31" s="20" t="n">
         <v>6000</v>
       </c>
-      <c r="Q28" s="20" t="n">
+      <c r="Q31" s="20" t="n">
         <v>6000</v>
       </c>
-      <c r="R28" s="20" t="n">
+      <c r="R31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="S28" s="20" t="n">
+      <c r="S31" s="20" t="n">
         <v>5000</v>
       </c>
-      <c r="T28" s="20" t="n">
+      <c r="T31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="U28" s="20" t="n">
+      <c r="U31" s="20" t="n">
         <v>8000</v>
       </c>
-      <c r="V28" s="20" t="n">
+      <c r="V31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="W28" s="20" t="n">
+      <c r="W31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="X28" s="20" t="n">
+      <c r="X31" s="20" t="n">
         <v>5000</v>
       </c>
-      <c r="Y28" s="20" t="n">
+      <c r="Y31" s="20" t="n">
         <v>6000</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">    Total Conference &amp; Travel</t>
         </is>
       </c>
-      <c r="B29" s="18">
-        <f>B28</f>
-        <v/>
-      </c>
-      <c r="C29" s="18">
-        <f>C28</f>
-        <v/>
-      </c>
-      <c r="D29" s="18">
-        <f>D28</f>
-        <v/>
-      </c>
-      <c r="E29" s="18">
-        <f>E28</f>
-        <v/>
-      </c>
-      <c r="F29" s="18">
-        <f>F28</f>
-        <v/>
-      </c>
-      <c r="G29" s="18">
-        <f>G28</f>
-        <v/>
-      </c>
-      <c r="H29" s="18">
-        <f>H28</f>
-        <v/>
-      </c>
-      <c r="I29" s="18">
-        <f>I28</f>
-        <v/>
-      </c>
-      <c r="J29" s="18">
-        <f>J28</f>
-        <v/>
-      </c>
-      <c r="K29" s="18">
-        <f>K28</f>
-        <v/>
-      </c>
-      <c r="L29" s="18">
-        <f>L28</f>
-        <v/>
-      </c>
-      <c r="M29" s="18">
-        <f>M28</f>
-        <v/>
-      </c>
-      <c r="N29" s="18">
-        <f>N28</f>
-        <v/>
-      </c>
-      <c r="O29" s="18">
-        <f>O28</f>
-        <v/>
-      </c>
-      <c r="P29" s="18">
-        <f>P28</f>
-        <v/>
-      </c>
-      <c r="Q29" s="18">
-        <f>Q28</f>
-        <v/>
-      </c>
-      <c r="R29" s="18">
-        <f>R28</f>
-        <v/>
-      </c>
-      <c r="S29" s="18">
-        <f>S28</f>
-        <v/>
-      </c>
-      <c r="T29" s="18">
-        <f>T28</f>
-        <v/>
-      </c>
-      <c r="U29" s="18">
-        <f>U28</f>
-        <v/>
-      </c>
-      <c r="V29" s="18">
-        <f>V28</f>
-        <v/>
-      </c>
-      <c r="W29" s="18">
-        <f>W28</f>
-        <v/>
-      </c>
-      <c r="X29" s="18">
-        <f>X28</f>
-        <v/>
-      </c>
-      <c r="Y29" s="18">
-        <f>Y28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="B32" s="18">
+        <f>B31</f>
+        <v/>
+      </c>
+      <c r="C32" s="18">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="D32" s="18">
+        <f>D31</f>
+        <v/>
+      </c>
+      <c r="E32" s="18">
+        <f>E31</f>
+        <v/>
+      </c>
+      <c r="F32" s="18">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="G32" s="18">
+        <f>G31</f>
+        <v/>
+      </c>
+      <c r="H32" s="18">
+        <f>H31</f>
+        <v/>
+      </c>
+      <c r="I32" s="18">
+        <f>I31</f>
+        <v/>
+      </c>
+      <c r="J32" s="18">
+        <f>J31</f>
+        <v/>
+      </c>
+      <c r="K32" s="18">
+        <f>K31</f>
+        <v/>
+      </c>
+      <c r="L32" s="18">
+        <f>L31</f>
+        <v/>
+      </c>
+      <c r="M32" s="18">
+        <f>M31</f>
+        <v/>
+      </c>
+      <c r="N32" s="18">
+        <f>N31</f>
+        <v/>
+      </c>
+      <c r="O32" s="18">
+        <f>O31</f>
+        <v/>
+      </c>
+      <c r="P32" s="18">
+        <f>P31</f>
+        <v/>
+      </c>
+      <c r="Q32" s="18">
+        <f>Q31</f>
+        <v/>
+      </c>
+      <c r="R32" s="18">
+        <f>R31</f>
+        <v/>
+      </c>
+      <c r="S32" s="18">
+        <f>S31</f>
+        <v/>
+      </c>
+      <c r="T32" s="18">
+        <f>T31</f>
+        <v/>
+      </c>
+      <c r="U32" s="18">
+        <f>U31</f>
+        <v/>
+      </c>
+      <c r="V32" s="18">
+        <f>V31</f>
+        <v/>
+      </c>
+      <c r="W32" s="18">
+        <f>W31</f>
+        <v/>
+      </c>
+      <c r="X32" s="18">
+        <f>X31</f>
+        <v/>
+      </c>
+      <c r="Y32" s="18">
+        <f>Y31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  TOTAL OPEX</t>
         </is>
       </c>
-      <c r="B31" s="18">
-        <f>B17+B25+B29</f>
-        <v/>
-      </c>
-      <c r="C31" s="18">
-        <f>C17+C25+C29</f>
-        <v/>
-      </c>
-      <c r="D31" s="18">
-        <f>D17+D25+D29</f>
-        <v/>
-      </c>
-      <c r="E31" s="18">
-        <f>E17+E25+E29</f>
-        <v/>
-      </c>
-      <c r="F31" s="18">
-        <f>F17+F25+F29</f>
-        <v/>
-      </c>
-      <c r="G31" s="18">
-        <f>G17+G25+G29</f>
-        <v/>
-      </c>
-      <c r="H31" s="18">
-        <f>H17+H25+H29</f>
-        <v/>
-      </c>
-      <c r="I31" s="18">
-        <f>I17+I25+I29</f>
-        <v/>
-      </c>
-      <c r="J31" s="18">
-        <f>J17+J25+J29</f>
-        <v/>
-      </c>
-      <c r="K31" s="18">
-        <f>K17+K25+K29</f>
-        <v/>
-      </c>
-      <c r="L31" s="18">
-        <f>L17+L25+L29</f>
-        <v/>
-      </c>
-      <c r="M31" s="18">
-        <f>M17+M25+M29</f>
-        <v/>
-      </c>
-      <c r="N31" s="18">
-        <f>N17+N25+N29</f>
-        <v/>
-      </c>
-      <c r="O31" s="18">
-        <f>O17+O25+O29</f>
-        <v/>
-      </c>
-      <c r="P31" s="18">
-        <f>P17+P25+P29</f>
-        <v/>
-      </c>
-      <c r="Q31" s="18">
-        <f>Q17+Q25+Q29</f>
-        <v/>
-      </c>
-      <c r="R31" s="18">
-        <f>R17+R25+R29</f>
-        <v/>
-      </c>
-      <c r="S31" s="18">
-        <f>S17+S25+S29</f>
-        <v/>
-      </c>
-      <c r="T31" s="18">
-        <f>T17+T25+T29</f>
-        <v/>
-      </c>
-      <c r="U31" s="18">
-        <f>U17+U25+U29</f>
-        <v/>
-      </c>
-      <c r="V31" s="18">
-        <f>V17+V25+V29</f>
-        <v/>
-      </c>
-      <c r="W31" s="18">
-        <f>W17+W25+W29</f>
-        <v/>
-      </c>
-      <c r="X31" s="18">
-        <f>X17+X25+X29</f>
-        <v/>
-      </c>
-      <c r="Y31" s="18">
-        <f>Y17+Y25+Y29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B33" s="18">
-        <f>B10-B31</f>
-        <v/>
-      </c>
-      <c r="C33" s="18">
-        <f>C10-C31</f>
-        <v/>
-      </c>
-      <c r="D33" s="18">
-        <f>D10-D31</f>
-        <v/>
-      </c>
-      <c r="E33" s="18">
-        <f>E10-E31</f>
-        <v/>
-      </c>
-      <c r="F33" s="18">
-        <f>F10-F31</f>
-        <v/>
-      </c>
-      <c r="G33" s="18">
-        <f>G10-G31</f>
-        <v/>
-      </c>
-      <c r="H33" s="18">
-        <f>H10-H31</f>
-        <v/>
-      </c>
-      <c r="I33" s="18">
-        <f>I10-I31</f>
-        <v/>
-      </c>
-      <c r="J33" s="18">
-        <f>J10-J31</f>
-        <v/>
-      </c>
-      <c r="K33" s="18">
-        <f>K10-K31</f>
-        <v/>
-      </c>
-      <c r="L33" s="18">
-        <f>L10-L31</f>
-        <v/>
-      </c>
-      <c r="M33" s="18">
-        <f>M10-M31</f>
-        <v/>
-      </c>
-      <c r="N33" s="18">
-        <f>N10-N31</f>
-        <v/>
-      </c>
-      <c r="O33" s="18">
-        <f>O10-O31</f>
-        <v/>
-      </c>
-      <c r="P33" s="18">
-        <f>P10-P31</f>
-        <v/>
-      </c>
-      <c r="Q33" s="18">
-        <f>Q10-Q31</f>
-        <v/>
-      </c>
-      <c r="R33" s="18">
-        <f>R10-R31</f>
-        <v/>
-      </c>
-      <c r="S33" s="18">
-        <f>S10-S31</f>
-        <v/>
-      </c>
-      <c r="T33" s="18">
-        <f>T10-T31</f>
-        <v/>
-      </c>
-      <c r="U33" s="18">
-        <f>U10-U31</f>
-        <v/>
-      </c>
-      <c r="V33" s="18">
-        <f>V10-V31</f>
-        <v/>
-      </c>
-      <c r="W33" s="18">
-        <f>W10-W31</f>
-        <v/>
-      </c>
-      <c r="X33" s="18">
-        <f>X10-X31</f>
-        <v/>
-      </c>
-      <c r="Y33" s="18">
-        <f>Y10-Y31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>EBITDA MARGIN %</t>
-        </is>
-      </c>
-      <c r="B34" s="16">
-        <f>IF(Revenue!B35&lt;&gt;0,B33/Revenue!B35,0)</f>
-        <v/>
-      </c>
-      <c r="C34" s="16">
-        <f>IF(Revenue!C35&lt;&gt;0,C33/Revenue!C35,0)</f>
-        <v/>
-      </c>
-      <c r="D34" s="16">
-        <f>IF(Revenue!D35&lt;&gt;0,D33/Revenue!D35,0)</f>
-        <v/>
-      </c>
-      <c r="E34" s="16">
-        <f>IF(Revenue!E35&lt;&gt;0,E33/Revenue!E35,0)</f>
-        <v/>
-      </c>
-      <c r="F34" s="16">
-        <f>IF(Revenue!F35&lt;&gt;0,F33/Revenue!F35,0)</f>
-        <v/>
-      </c>
-      <c r="G34" s="16">
-        <f>IF(Revenue!G35&lt;&gt;0,G33/Revenue!G35,0)</f>
-        <v/>
-      </c>
-      <c r="H34" s="16">
-        <f>IF(Revenue!H35&lt;&gt;0,H33/Revenue!H35,0)</f>
-        <v/>
-      </c>
-      <c r="I34" s="16">
-        <f>IF(Revenue!I35&lt;&gt;0,I33/Revenue!I35,0)</f>
-        <v/>
-      </c>
-      <c r="J34" s="16">
-        <f>IF(Revenue!J35&lt;&gt;0,J33/Revenue!J35,0)</f>
-        <v/>
-      </c>
-      <c r="K34" s="16">
-        <f>IF(Revenue!K35&lt;&gt;0,K33/Revenue!K35,0)</f>
-        <v/>
-      </c>
-      <c r="L34" s="16">
-        <f>IF(Revenue!L35&lt;&gt;0,L33/Revenue!L35,0)</f>
-        <v/>
-      </c>
-      <c r="M34" s="16">
-        <f>IF(Revenue!M35&lt;&gt;0,M33/Revenue!M35,0)</f>
-        <v/>
-      </c>
-      <c r="N34" s="16">
-        <f>IF(Revenue!N35&lt;&gt;0,N33/Revenue!N35,0)</f>
-        <v/>
-      </c>
-      <c r="O34" s="16">
-        <f>IF(Revenue!O35&lt;&gt;0,O33/Revenue!O35,0)</f>
-        <v/>
-      </c>
-      <c r="P34" s="16">
-        <f>IF(Revenue!P35&lt;&gt;0,P33/Revenue!P35,0)</f>
-        <v/>
-      </c>
-      <c r="Q34" s="16">
-        <f>IF(Revenue!Q35&lt;&gt;0,Q33/Revenue!Q35,0)</f>
-        <v/>
-      </c>
-      <c r="R34" s="16">
-        <f>IF(Revenue!R35&lt;&gt;0,R33/Revenue!R35,0)</f>
-        <v/>
-      </c>
-      <c r="S34" s="16">
-        <f>IF(Revenue!S35&lt;&gt;0,S33/Revenue!S35,0)</f>
-        <v/>
-      </c>
-      <c r="T34" s="16">
-        <f>IF(Revenue!T35&lt;&gt;0,T33/Revenue!T35,0)</f>
-        <v/>
-      </c>
-      <c r="U34" s="16">
-        <f>IF(Revenue!U35&lt;&gt;0,U33/Revenue!U35,0)</f>
-        <v/>
-      </c>
-      <c r="V34" s="16">
-        <f>IF(Revenue!V35&lt;&gt;0,V33/Revenue!V35,0)</f>
-        <v/>
-      </c>
-      <c r="W34" s="16">
-        <f>IF(Revenue!W35&lt;&gt;0,W33/Revenue!W35,0)</f>
-        <v/>
-      </c>
-      <c r="X34" s="16">
-        <f>IF(Revenue!X35&lt;&gt;0,X33/Revenue!X35,0)</f>
-        <v/>
-      </c>
-      <c r="Y34" s="16">
-        <f>IF(Revenue!Y35&lt;&gt;0,Y33/Revenue!Y35,0)</f>
+      <c r="B34" s="18">
+        <f>B17+B28+B32</f>
+        <v/>
+      </c>
+      <c r="C34" s="18">
+        <f>C17+C28+C32</f>
+        <v/>
+      </c>
+      <c r="D34" s="18">
+        <f>D17+D28+D32</f>
+        <v/>
+      </c>
+      <c r="E34" s="18">
+        <f>E17+E28+E32</f>
+        <v/>
+      </c>
+      <c r="F34" s="18">
+        <f>F17+F28+F32</f>
+        <v/>
+      </c>
+      <c r="G34" s="18">
+        <f>G17+G28+G32</f>
+        <v/>
+      </c>
+      <c r="H34" s="18">
+        <f>H17+H28+H32</f>
+        <v/>
+      </c>
+      <c r="I34" s="18">
+        <f>I17+I28+I32</f>
+        <v/>
+      </c>
+      <c r="J34" s="18">
+        <f>J17+J28+J32</f>
+        <v/>
+      </c>
+      <c r="K34" s="18">
+        <f>K17+K28+K32</f>
+        <v/>
+      </c>
+      <c r="L34" s="18">
+        <f>L17+L28+L32</f>
+        <v/>
+      </c>
+      <c r="M34" s="18">
+        <f>M17+M28+M32</f>
+        <v/>
+      </c>
+      <c r="N34" s="18">
+        <f>N17+N28+N32</f>
+        <v/>
+      </c>
+      <c r="O34" s="18">
+        <f>O17+O28+O32</f>
+        <v/>
+      </c>
+      <c r="P34" s="18">
+        <f>P17+P28+P32</f>
+        <v/>
+      </c>
+      <c r="Q34" s="18">
+        <f>Q17+Q28+Q32</f>
+        <v/>
+      </c>
+      <c r="R34" s="18">
+        <f>R17+R28+R32</f>
+        <v/>
+      </c>
+      <c r="S34" s="18">
+        <f>S17+S28+S32</f>
+        <v/>
+      </c>
+      <c r="T34" s="18">
+        <f>T17+T28+T32</f>
+        <v/>
+      </c>
+      <c r="U34" s="18">
+        <f>U17+U28+U32</f>
+        <v/>
+      </c>
+      <c r="V34" s="18">
+        <f>V17+V28+V32</f>
+        <v/>
+      </c>
+      <c r="W34" s="18">
+        <f>W17+W28+W32</f>
+        <v/>
+      </c>
+      <c r="X34" s="18">
+        <f>X17+X28+X32</f>
+        <v/>
+      </c>
+      <c r="Y34" s="18">
+        <f>Y17+Y28+Y32</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B36" s="18">
+        <f>B10-B34</f>
+        <v/>
+      </c>
+      <c r="C36" s="18">
+        <f>C10-C34</f>
+        <v/>
+      </c>
+      <c r="D36" s="18">
+        <f>D10-D34</f>
+        <v/>
+      </c>
+      <c r="E36" s="18">
+        <f>E10-E34</f>
+        <v/>
+      </c>
+      <c r="F36" s="18">
+        <f>F10-F34</f>
+        <v/>
+      </c>
+      <c r="G36" s="18">
+        <f>G10-G34</f>
+        <v/>
+      </c>
+      <c r="H36" s="18">
+        <f>H10-H34</f>
+        <v/>
+      </c>
+      <c r="I36" s="18">
+        <f>I10-I34</f>
+        <v/>
+      </c>
+      <c r="J36" s="18">
+        <f>J10-J34</f>
+        <v/>
+      </c>
+      <c r="K36" s="18">
+        <f>K10-K34</f>
+        <v/>
+      </c>
+      <c r="L36" s="18">
+        <f>L10-L34</f>
+        <v/>
+      </c>
+      <c r="M36" s="18">
+        <f>M10-M34</f>
+        <v/>
+      </c>
+      <c r="N36" s="18">
+        <f>N10-N34</f>
+        <v/>
+      </c>
+      <c r="O36" s="18">
+        <f>O10-O34</f>
+        <v/>
+      </c>
+      <c r="P36" s="18">
+        <f>P10-P34</f>
+        <v/>
+      </c>
+      <c r="Q36" s="18">
+        <f>Q10-Q34</f>
+        <v/>
+      </c>
+      <c r="R36" s="18">
+        <f>R10-R34</f>
+        <v/>
+      </c>
+      <c r="S36" s="18">
+        <f>S10-S34</f>
+        <v/>
+      </c>
+      <c r="T36" s="18">
+        <f>T10-T34</f>
+        <v/>
+      </c>
+      <c r="U36" s="18">
+        <f>U10-U34</f>
+        <v/>
+      </c>
+      <c r="V36" s="18">
+        <f>V10-V34</f>
+        <v/>
+      </c>
+      <c r="W36" s="18">
+        <f>W10-W34</f>
+        <v/>
+      </c>
+      <c r="X36" s="18">
+        <f>X10-X34</f>
+        <v/>
+      </c>
+      <c r="Y36" s="18">
+        <f>Y10-Y34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>EBITDA MARGIN %</t>
+        </is>
+      </c>
+      <c r="B37" s="16">
+        <f>IF(Revenue!B35&lt;&gt;0,B36/Revenue!B35,0)</f>
+        <v/>
+      </c>
+      <c r="C37" s="16">
+        <f>IF(Revenue!C35&lt;&gt;0,C36/Revenue!C35,0)</f>
+        <v/>
+      </c>
+      <c r="D37" s="16">
+        <f>IF(Revenue!D35&lt;&gt;0,D36/Revenue!D35,0)</f>
+        <v/>
+      </c>
+      <c r="E37" s="16">
+        <f>IF(Revenue!E35&lt;&gt;0,E36/Revenue!E35,0)</f>
+        <v/>
+      </c>
+      <c r="F37" s="16">
+        <f>IF(Revenue!F35&lt;&gt;0,F36/Revenue!F35,0)</f>
+        <v/>
+      </c>
+      <c r="G37" s="16">
+        <f>IF(Revenue!G35&lt;&gt;0,G36/Revenue!G35,0)</f>
+        <v/>
+      </c>
+      <c r="H37" s="16">
+        <f>IF(Revenue!H35&lt;&gt;0,H36/Revenue!H35,0)</f>
+        <v/>
+      </c>
+      <c r="I37" s="16">
+        <f>IF(Revenue!I35&lt;&gt;0,I36/Revenue!I35,0)</f>
+        <v/>
+      </c>
+      <c r="J37" s="16">
+        <f>IF(Revenue!J35&lt;&gt;0,J36/Revenue!J35,0)</f>
+        <v/>
+      </c>
+      <c r="K37" s="16">
+        <f>IF(Revenue!K35&lt;&gt;0,K36/Revenue!K35,0)</f>
+        <v/>
+      </c>
+      <c r="L37" s="16">
+        <f>IF(Revenue!L35&lt;&gt;0,L36/Revenue!L35,0)</f>
+        <v/>
+      </c>
+      <c r="M37" s="16">
+        <f>IF(Revenue!M35&lt;&gt;0,M36/Revenue!M35,0)</f>
+        <v/>
+      </c>
+      <c r="N37" s="16">
+        <f>IF(Revenue!N35&lt;&gt;0,N36/Revenue!N35,0)</f>
+        <v/>
+      </c>
+      <c r="O37" s="16">
+        <f>IF(Revenue!O35&lt;&gt;0,O36/Revenue!O35,0)</f>
+        <v/>
+      </c>
+      <c r="P37" s="16">
+        <f>IF(Revenue!P35&lt;&gt;0,P36/Revenue!P35,0)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="16">
+        <f>IF(Revenue!Q35&lt;&gt;0,Q36/Revenue!Q35,0)</f>
+        <v/>
+      </c>
+      <c r="R37" s="16">
+        <f>IF(Revenue!R35&lt;&gt;0,R36/Revenue!R35,0)</f>
+        <v/>
+      </c>
+      <c r="S37" s="16">
+        <f>IF(Revenue!S35&lt;&gt;0,S36/Revenue!S35,0)</f>
+        <v/>
+      </c>
+      <c r="T37" s="16">
+        <f>IF(Revenue!T35&lt;&gt;0,T36/Revenue!T35,0)</f>
+        <v/>
+      </c>
+      <c r="U37" s="16">
+        <f>IF(Revenue!U35&lt;&gt;0,U36/Revenue!U35,0)</f>
+        <v/>
+      </c>
+      <c r="V37" s="16">
+        <f>IF(Revenue!V35&lt;&gt;0,V36/Revenue!V35,0)</f>
+        <v/>
+      </c>
+      <c r="W37" s="16">
+        <f>IF(Revenue!W35&lt;&gt;0,W36/Revenue!W35,0)</f>
+        <v/>
+      </c>
+      <c r="X37" s="16">
+        <f>IF(Revenue!X35&lt;&gt;0,X36/Revenue!X35,0)</f>
+        <v/>
+      </c>
+      <c r="Y37" s="16">
+        <f>IF(Revenue!Y35&lt;&gt;0,Y36/Revenue!Y35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
           <t>NET INCOME</t>
         </is>
       </c>
-      <c r="B36" s="18">
-        <f>B33</f>
-        <v/>
-      </c>
-      <c r="C36" s="18">
-        <f>C33</f>
-        <v/>
-      </c>
-      <c r="D36" s="18">
-        <f>D33</f>
-        <v/>
-      </c>
-      <c r="E36" s="18">
-        <f>E33</f>
-        <v/>
-      </c>
-      <c r="F36" s="18">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="G36" s="18">
-        <f>G33</f>
-        <v/>
-      </c>
-      <c r="H36" s="18">
-        <f>H33</f>
-        <v/>
-      </c>
-      <c r="I36" s="18">
-        <f>I33</f>
-        <v/>
-      </c>
-      <c r="J36" s="18">
-        <f>J33</f>
-        <v/>
-      </c>
-      <c r="K36" s="18">
-        <f>K33</f>
-        <v/>
-      </c>
-      <c r="L36" s="18">
-        <f>L33</f>
-        <v/>
-      </c>
-      <c r="M36" s="18">
-        <f>M33</f>
-        <v/>
-      </c>
-      <c r="N36" s="18">
-        <f>N33</f>
-        <v/>
-      </c>
-      <c r="O36" s="18">
-        <f>O33</f>
-        <v/>
-      </c>
-      <c r="P36" s="18">
-        <f>P33</f>
-        <v/>
-      </c>
-      <c r="Q36" s="18">
-        <f>Q33</f>
-        <v/>
-      </c>
-      <c r="R36" s="18">
-        <f>R33</f>
-        <v/>
-      </c>
-      <c r="S36" s="18">
-        <f>S33</f>
-        <v/>
-      </c>
-      <c r="T36" s="18">
-        <f>T33</f>
-        <v/>
-      </c>
-      <c r="U36" s="18">
-        <f>U33</f>
-        <v/>
-      </c>
-      <c r="V36" s="18">
-        <f>V33</f>
-        <v/>
-      </c>
-      <c r="W36" s="18">
-        <f>W33</f>
-        <v/>
-      </c>
-      <c r="X36" s="18">
-        <f>X33</f>
-        <v/>
-      </c>
-      <c r="Y36" s="18">
-        <f>Y33</f>
+      <c r="B39" s="18">
+        <f>B36</f>
+        <v/>
+      </c>
+      <c r="C39" s="18">
+        <f>C36</f>
+        <v/>
+      </c>
+      <c r="D39" s="18">
+        <f>D36</f>
+        <v/>
+      </c>
+      <c r="E39" s="18">
+        <f>E36</f>
+        <v/>
+      </c>
+      <c r="F39" s="18">
+        <f>F36</f>
+        <v/>
+      </c>
+      <c r="G39" s="18">
+        <f>G36</f>
+        <v/>
+      </c>
+      <c r="H39" s="18">
+        <f>H36</f>
+        <v/>
+      </c>
+      <c r="I39" s="18">
+        <f>I36</f>
+        <v/>
+      </c>
+      <c r="J39" s="18">
+        <f>J36</f>
+        <v/>
+      </c>
+      <c r="K39" s="18">
+        <f>K36</f>
+        <v/>
+      </c>
+      <c r="L39" s="18">
+        <f>L36</f>
+        <v/>
+      </c>
+      <c r="M39" s="18">
+        <f>M36</f>
+        <v/>
+      </c>
+      <c r="N39" s="18">
+        <f>N36</f>
+        <v/>
+      </c>
+      <c r="O39" s="18">
+        <f>O36</f>
+        <v/>
+      </c>
+      <c r="P39" s="18">
+        <f>P36</f>
+        <v/>
+      </c>
+      <c r="Q39" s="18">
+        <f>Q36</f>
+        <v/>
+      </c>
+      <c r="R39" s="18">
+        <f>R36</f>
+        <v/>
+      </c>
+      <c r="S39" s="18">
+        <f>S36</f>
+        <v/>
+      </c>
+      <c r="T39" s="18">
+        <f>T36</f>
+        <v/>
+      </c>
+      <c r="U39" s="18">
+        <f>U36</f>
+        <v/>
+      </c>
+      <c r="V39" s="18">
+        <f>V36</f>
+        <v/>
+      </c>
+      <c r="W39" s="18">
+        <f>W36</f>
+        <v/>
+      </c>
+      <c r="X39" s="18">
+        <f>X36</f>
+        <v/>
+      </c>
+      <c r="Y39" s="18">
+        <f>Y36</f>
         <v/>
       </c>
     </row>
@@ -11168,7 +12447,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33:Y33">
+  <conditionalFormatting sqref="B36:Y36">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -11176,7 +12455,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B36:Y36">
+  <conditionalFormatting sqref="B39:Y39">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -12556,7 +13835,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Assumptions!$B$147</f>
+        <f>Assumptions!$B$200</f>
         <v/>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -12590,99 +13869,99 @@
         </is>
       </c>
       <c r="B3" s="15">
-        <f>'COGS &amp; Operating Expenses'!B33</f>
+        <f>'COGS &amp; Operating Expenses'!B36</f>
         <v/>
       </c>
       <c r="C3" s="15">
-        <f>'COGS &amp; Operating Expenses'!C33</f>
+        <f>'COGS &amp; Operating Expenses'!C36</f>
         <v/>
       </c>
       <c r="D3" s="15">
-        <f>'COGS &amp; Operating Expenses'!D33</f>
+        <f>'COGS &amp; Operating Expenses'!D36</f>
         <v/>
       </c>
       <c r="E3" s="15">
-        <f>'COGS &amp; Operating Expenses'!E33</f>
+        <f>'COGS &amp; Operating Expenses'!E36</f>
         <v/>
       </c>
       <c r="F3" s="15">
-        <f>'COGS &amp; Operating Expenses'!F33</f>
+        <f>'COGS &amp; Operating Expenses'!F36</f>
         <v/>
       </c>
       <c r="G3" s="15">
-        <f>'COGS &amp; Operating Expenses'!G33</f>
+        <f>'COGS &amp; Operating Expenses'!G36</f>
         <v/>
       </c>
       <c r="H3" s="15">
-        <f>'COGS &amp; Operating Expenses'!H33</f>
+        <f>'COGS &amp; Operating Expenses'!H36</f>
         <v/>
       </c>
       <c r="I3" s="15">
-        <f>'COGS &amp; Operating Expenses'!I33</f>
+        <f>'COGS &amp; Operating Expenses'!I36</f>
         <v/>
       </c>
       <c r="J3" s="15">
-        <f>'COGS &amp; Operating Expenses'!J33</f>
+        <f>'COGS &amp; Operating Expenses'!J36</f>
         <v/>
       </c>
       <c r="K3" s="15">
-        <f>'COGS &amp; Operating Expenses'!K33</f>
+        <f>'COGS &amp; Operating Expenses'!K36</f>
         <v/>
       </c>
       <c r="L3" s="15">
-        <f>'COGS &amp; Operating Expenses'!L33</f>
+        <f>'COGS &amp; Operating Expenses'!L36</f>
         <v/>
       </c>
       <c r="M3" s="15">
-        <f>'COGS &amp; Operating Expenses'!M33</f>
+        <f>'COGS &amp; Operating Expenses'!M36</f>
         <v/>
       </c>
       <c r="N3" s="15">
-        <f>'COGS &amp; Operating Expenses'!N33</f>
+        <f>'COGS &amp; Operating Expenses'!N36</f>
         <v/>
       </c>
       <c r="O3" s="15">
-        <f>'COGS &amp; Operating Expenses'!O33</f>
+        <f>'COGS &amp; Operating Expenses'!O36</f>
         <v/>
       </c>
       <c r="P3" s="15">
-        <f>'COGS &amp; Operating Expenses'!P33</f>
+        <f>'COGS &amp; Operating Expenses'!P36</f>
         <v/>
       </c>
       <c r="Q3" s="15">
-        <f>'COGS &amp; Operating Expenses'!Q33</f>
+        <f>'COGS &amp; Operating Expenses'!Q36</f>
         <v/>
       </c>
       <c r="R3" s="15">
-        <f>'COGS &amp; Operating Expenses'!R33</f>
+        <f>'COGS &amp; Operating Expenses'!R36</f>
         <v/>
       </c>
       <c r="S3" s="15">
-        <f>'COGS &amp; Operating Expenses'!S33</f>
+        <f>'COGS &amp; Operating Expenses'!S36</f>
         <v/>
       </c>
       <c r="T3" s="15">
-        <f>'COGS &amp; Operating Expenses'!T33</f>
+        <f>'COGS &amp; Operating Expenses'!T36</f>
         <v/>
       </c>
       <c r="U3" s="15">
-        <f>'COGS &amp; Operating Expenses'!U33</f>
+        <f>'COGS &amp; Operating Expenses'!U36</f>
         <v/>
       </c>
       <c r="V3" s="15">
-        <f>'COGS &amp; Operating Expenses'!V33</f>
+        <f>'COGS &amp; Operating Expenses'!V36</f>
         <v/>
       </c>
       <c r="W3" s="15">
-        <f>'COGS &amp; Operating Expenses'!W33</f>
+        <f>'COGS &amp; Operating Expenses'!W36</f>
         <v/>
       </c>
       <c r="X3" s="15">
-        <f>'COGS &amp; Operating Expenses'!X33</f>
+        <f>'COGS &amp; Operating Expenses'!X36</f>
         <v/>
       </c>
       <c r="Y3" s="15">
-        <f>'COGS &amp; Operating Expenses'!Y33</f>
+        <f>'COGS &amp; Operating Expenses'!Y36</f>
         <v/>
       </c>
     </row>
@@ -12693,7 +13972,7 @@
         </is>
       </c>
       <c r="B4" s="18">
-        <f>Assumptions!$B$147+B3</f>
+        <f>Assumptions!$B$200+B3</f>
         <v/>
       </c>
       <c r="C4" s="18">
@@ -13030,7 +14309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -13332,7 +14611,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>DFS Regulatory / Licensing</t>
+          <t>DFS Regulatory — Canada</t>
         </is>
       </c>
       <c r="B20" s="15">
@@ -13351,15 +14630,15 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Total OPEX</t>
+          <t>US DFS Expansion (Total)</t>
         </is>
       </c>
       <c r="B21" s="15">
-        <f>SUM('COGS &amp; Operating Expenses'!B31:'COGS &amp; Operating Expenses'!M31)</f>
+        <f>SUM('COGS &amp; Operating Expenses'!B25:'COGS &amp; Operating Expenses'!M25)</f>
         <v/>
       </c>
       <c r="C21" s="15">
-        <f>SUM('COGS &amp; Operating Expenses'!N31:'COGS &amp; Operating Expenses'!Y31)</f>
+        <f>SUM('COGS &amp; Operating Expenses'!N25:'COGS &amp; Operating Expenses'!Y25)</f>
         <v/>
       </c>
       <c r="D21" s="16">
@@ -13370,15 +14649,15 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>EBITDA / Net Income</t>
+          <t>Total OPEX</t>
         </is>
       </c>
       <c r="B22" s="15">
-        <f>SUM('COGS &amp; Operating Expenses'!B33:'COGS &amp; Operating Expenses'!M33)</f>
+        <f>SUM('COGS &amp; Operating Expenses'!B34:'COGS &amp; Operating Expenses'!M34)</f>
         <v/>
       </c>
       <c r="C22" s="15">
-        <f>SUM('COGS &amp; Operating Expenses'!N33:'COGS &amp; Operating Expenses'!Y33)</f>
+        <f>SUM('COGS &amp; Operating Expenses'!N34:'COGS &amp; Operating Expenses'!Y34)</f>
         <v/>
       </c>
       <c r="D22" s="16">
@@ -13386,45 +14665,64 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>EBITDA / Net Income</t>
+        </is>
+      </c>
+      <c r="B23" s="15">
+        <f>SUM('COGS &amp; Operating Expenses'!B36:'COGS &amp; Operating Expenses'!M36)</f>
+        <v/>
+      </c>
+      <c r="C23" s="15">
+        <f>SUM('COGS &amp; Operating Expenses'!N36:'COGS &amp; Operating Expenses'!Y36)</f>
+        <v/>
+      </c>
+      <c r="D23" s="16">
+        <f>IF(ABS(B23)&gt;0,(C23-B23)/ABS(B23),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>MARGINS</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Gross Margin %</t>
-        </is>
-      </c>
-      <c r="B25" s="16">
-        <f>IF(B14&lt;&gt;0,B18/B14,0)</f>
-        <v/>
-      </c>
-      <c r="C25" s="16">
-        <f>IF(C14&lt;&gt;0,C18/C14,0)</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>Gross Margin %</t>
+        </is>
+      </c>
+      <c r="B26" s="16">
+        <f>IF(B14&lt;&gt;0,B18/B14,0)</f>
+        <v/>
+      </c>
+      <c r="C26" s="16">
+        <f>IF(C14&lt;&gt;0,C18/C14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>EBITDA Margin %</t>
         </is>
       </c>
-      <c r="B26" s="16">
-        <f>IF(B14&lt;&gt;0,B22/B14,0)</f>
-        <v/>
-      </c>
-      <c r="C26" s="16">
-        <f>IF(C14&lt;&gt;0,C22/C14,0)</f>
+      <c r="B27" s="16">
+        <f>IF(B14&lt;&gt;0,B23/B14,0)</f>
+        <v/>
+      </c>
+      <c r="C27" s="16">
+        <f>IF(C14&lt;&gt;0,C23/C14,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B22:C22">
+  <conditionalFormatting sqref="B23:C23">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -13865,7 +15163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -14582,7 +15880,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>DYNAMIC MODEL NOTE</t>
+          <t>US DFS EXPANSION (TOGGLE — SET TO 99 = OFF)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -14590,34 +15888,174 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>All computed cells use Excel formulas</t>
+          <t>NY Gaming Commission — $500K Y1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Change any yellow input cell to recalculate instantly</t>
+          <t>Most expensive US state for DFS</t>
+        </is>
+      </c>
+      <c r="C60" s="28" t="inlineStr">
+        <is>
+          <t>https://www.gaming.ny.gov/fantasysports</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Input cells on Assumptions tab</t>
+          <t>State-by-state licensing fees</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>All model inputs: pricing, rates, costs, AND monthly new user targets</t>
+          <t>19 states with DFS registration/licensing</t>
+        </is>
+      </c>
+      <c r="C61" s="28" t="inlineStr">
+        <is>
+          <t>https://www.legalsportsreport.com/dfs-bill-tracker/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>GeoComply geolocation vendor</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Required for multi-state compliance</t>
+        </is>
+      </c>
+      <c r="C62" s="28" t="inlineStr">
+        <is>
+          <t>https://www.geocomply.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>NY DFS revenue tax ~15%</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Tax on DFS revenue from NY users</t>
+        </is>
+      </c>
+      <c r="C63" s="28" t="inlineStr">
+        <is>
+          <t>https://www.gaming.ny.gov/fantasysports</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Estimated all-state Y1 cost ~$850K</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Licensing fees only; +$285K/yr compliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>METHODOLOGY NOTES (continued)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>US DFS expansion toggle</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Set month index on Assumptions tab (99 = OFF); Y1 fees amortized /12, then annual renewal /12</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>US DFS states modeled (19)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>NY, MA, VA, TN, IN, PA, CT, CO, IL, MO, OR, MD, KS, VT, AR, MS, NH, DE, RI</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>US banned states</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Idaho, Hawaii banned; Nevada requires full gaming license (~$500K+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>DYNAMIC MODEL NOTE</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>All computed cells use Excel formulas</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Change any yellow input cell to recalculate instantly</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Input cells on Assumptions tab</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>All model inputs: pricing, rates, costs, AND monthly new user targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>Input cells on COGS tab</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>Monthly conference/travel costs</t>
         </is>

</xml_diff>

<commit_message>
Gate monthly subscriptions and DFS revenue to in-season only
Monthly billing (Pro + Commissioner) now shows $0 during off-season months —
only annual billing subscribers continue generating revenue year-round.
DFS revenue is also gated on in-season in addition to the launch month check.

https://claude.ai/code/session_01DWcMBbfjeLfgrVr7i298sA
</commit_message>
<xml_diff>
--- a/docs/Citrus_Business_Model.xlsx
+++ b/docs/Citrus_Business_Model.xlsx
@@ -6458,99 +6458,99 @@
         </is>
       </c>
       <c r="B3" s="15">
-        <f>'User Growth'!B18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!B2="IN-SEASON",'User Growth'!B18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="C3" s="15">
-        <f>'User Growth'!C18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!C2="IN-SEASON",'User Growth'!C18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="D3" s="15">
-        <f>'User Growth'!D18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!D2="IN-SEASON",'User Growth'!D18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="E3" s="15">
-        <f>'User Growth'!E18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!E2="IN-SEASON",'User Growth'!E18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="F3" s="15">
-        <f>'User Growth'!F18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!F2="IN-SEASON",'User Growth'!F18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="G3" s="15">
-        <f>'User Growth'!G18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!G2="IN-SEASON",'User Growth'!G18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="H3" s="15">
-        <f>'User Growth'!H18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!H2="IN-SEASON",'User Growth'!H18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="I3" s="15">
-        <f>'User Growth'!I18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!I2="IN-SEASON",'User Growth'!I18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="J3" s="15">
-        <f>'User Growth'!J18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!J2="IN-SEASON",'User Growth'!J18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="K3" s="15">
-        <f>'User Growth'!K18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!K2="IN-SEASON",'User Growth'!K18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="L3" s="15">
-        <f>'User Growth'!L18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!L2="IN-SEASON",'User Growth'!L18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="M3" s="15">
-        <f>'User Growth'!M18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!M2="IN-SEASON",'User Growth'!M18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="N3" s="15">
-        <f>'User Growth'!N18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!N2="IN-SEASON",'User Growth'!N18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="O3" s="15">
-        <f>'User Growth'!O18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!O2="IN-SEASON",'User Growth'!O18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="P3" s="15">
-        <f>'User Growth'!P18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!P2="IN-SEASON",'User Growth'!P18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="Q3" s="15">
-        <f>'User Growth'!Q18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!Q2="IN-SEASON",'User Growth'!Q18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="R3" s="15">
-        <f>'User Growth'!R18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!R2="IN-SEASON",'User Growth'!R18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="S3" s="15">
-        <f>'User Growth'!S18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!S2="IN-SEASON",'User Growth'!S18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="T3" s="15">
-        <f>'User Growth'!T18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!T2="IN-SEASON",'User Growth'!T18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="U3" s="15">
-        <f>'User Growth'!U18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!U2="IN-SEASON",'User Growth'!U18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="V3" s="15">
-        <f>'User Growth'!V18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!V2="IN-SEASON",'User Growth'!V18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="W3" s="15">
-        <f>'User Growth'!W18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!W2="IN-SEASON",'User Growth'!W18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="X3" s="15">
-        <f>'User Growth'!X18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!X2="IN-SEASON",'User Growth'!X18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
       <c r="Y3" s="15">
-        <f>'User Growth'!Y18*Assumptions!$B$7*Assumptions!$B$3</f>
+        <f>IF('User Growth'!Y2="IN-SEASON",'User Growth'!Y18*Assumptions!$B$7*Assumptions!$B$3,0)</f>
         <v/>
       </c>
     </row>
@@ -6664,99 +6664,99 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>'User Growth'!B19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!B2="IN-SEASON",'User Growth'!B19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="C5" s="15">
-        <f>'User Growth'!C19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!C2="IN-SEASON",'User Growth'!C19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="D5" s="15">
-        <f>'User Growth'!D19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!D2="IN-SEASON",'User Growth'!D19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>'User Growth'!E19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!E2="IN-SEASON",'User Growth'!E19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="F5" s="15">
-        <f>'User Growth'!F19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!F2="IN-SEASON",'User Growth'!F19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="G5" s="15">
-        <f>'User Growth'!G19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!G2="IN-SEASON",'User Growth'!G19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="H5" s="15">
-        <f>'User Growth'!H19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!H2="IN-SEASON",'User Growth'!H19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="I5" s="15">
-        <f>'User Growth'!I19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!I2="IN-SEASON",'User Growth'!I19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="J5" s="15">
-        <f>'User Growth'!J19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!J2="IN-SEASON",'User Growth'!J19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="K5" s="15">
-        <f>'User Growth'!K19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!K2="IN-SEASON",'User Growth'!K19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="L5" s="15">
-        <f>'User Growth'!L19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!L2="IN-SEASON",'User Growth'!L19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="M5" s="15">
-        <f>'User Growth'!M19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!M2="IN-SEASON",'User Growth'!M19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="N5" s="15">
-        <f>'User Growth'!N19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!N2="IN-SEASON",'User Growth'!N19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="O5" s="15">
-        <f>'User Growth'!O19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!O2="IN-SEASON",'User Growth'!O19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="P5" s="15">
-        <f>'User Growth'!P19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!P2="IN-SEASON",'User Growth'!P19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="Q5" s="15">
-        <f>'User Growth'!Q19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!Q2="IN-SEASON",'User Growth'!Q19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="R5" s="15">
-        <f>'User Growth'!R19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!R2="IN-SEASON",'User Growth'!R19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="S5" s="15">
-        <f>'User Growth'!S19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!S2="IN-SEASON",'User Growth'!S19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="T5" s="15">
-        <f>'User Growth'!T19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!T2="IN-SEASON",'User Growth'!T19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="U5" s="15">
-        <f>'User Growth'!U19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!U2="IN-SEASON",'User Growth'!U19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="V5" s="15">
-        <f>'User Growth'!V19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!V2="IN-SEASON",'User Growth'!V19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="W5" s="15">
-        <f>'User Growth'!W19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!W2="IN-SEASON",'User Growth'!W19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="X5" s="15">
-        <f>'User Growth'!X19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!X2="IN-SEASON",'User Growth'!X19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
       <c r="Y5" s="15">
-        <f>'User Growth'!Y19*Assumptions!$B$7*Assumptions!$B$4</f>
+        <f>IF('User Growth'!Y2="IN-SEASON",'User Growth'!Y19*Assumptions!$B$7*Assumptions!$B$4,0)</f>
         <v/>
       </c>
     </row>
@@ -7605,99 +7605,99 @@
         </is>
       </c>
       <c r="B18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!B20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!B2="IN-SEASON"),'User Growth'!B20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="C18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!C20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!C2="IN-SEASON"),'User Growth'!C20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="D18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!D20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!D2="IN-SEASON"),'User Growth'!D20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="E18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!E20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!E2="IN-SEASON"),'User Growth'!E20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="F18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!F20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!F2="IN-SEASON"),'User Growth'!F20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="G18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!G20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!G2="IN-SEASON"),'User Growth'!G20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="H18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!H20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!H2="IN-SEASON"),'User Growth'!H20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="I18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!I20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!I2="IN-SEASON"),'User Growth'!I20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="J18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!J20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!J2="IN-SEASON"),'User Growth'!J20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="K18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!K20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!K2="IN-SEASON"),'User Growth'!K20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="L18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!L20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!L2="IN-SEASON"),'User Growth'!L20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="M18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!M20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!M2="IN-SEASON"),'User Growth'!M20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="N18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!N20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!N2="IN-SEASON"),'User Growth'!N20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="O18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!O20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!O2="IN-SEASON"),'User Growth'!O20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="P18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!P20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!P2="IN-SEASON"),'User Growth'!P20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="Q18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!Q20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!Q2="IN-SEASON"),'User Growth'!Q20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="R18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!R20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!R2="IN-SEASON"),'User Growth'!R20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="S18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!S20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!S2="IN-SEASON"),'User Growth'!S20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="T18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!T20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!T2="IN-SEASON"),'User Growth'!T20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="U18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!U20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!U2="IN-SEASON"),'User Growth'!U20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="V18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!V20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!V2="IN-SEASON"),'User Growth'!V20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="W18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!W20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!W2="IN-SEASON"),'User Growth'!W20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="X18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!X20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!X2="IN-SEASON"),'User Growth'!X20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
       <c r="Y18" s="15">
-        <f>IF(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!Y20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
+        <f>IF(AND(COLUMN()-2&gt;=Assumptions!$B$44,'User Growth'!Y2="IN-SEASON"),'User Growth'!Y20*Assumptions!$B$42*Assumptions!$B$43*Assumptions!$B$41,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>